<commit_message>
Fix: history-hint exige anafora clara, no arrastra recurso
</commit_message>
<xml_diff>
--- a/Pulso_AI_matriz_evaluacion.xlsx
+++ b/Pulso_AI_matriz_evaluacion.xlsx
@@ -770,10 +770,6 @@
           <t>Recuento final (sobre 55 preguntas)</t>
         </is>
       </c>
-      <c r="C5" s="29" t="n"/>
-      <c r="D5" s="29" t="n"/>
-      <c r="E5" s="29" t="n"/>
-      <c r="F5" s="29" t="n"/>
     </row>
     <row r="6" ht="40" customHeight="1">
       <c r="B6" s="30" t="inlineStr">
@@ -832,10 +828,6 @@
           <t>Los 6 bugs raíz</t>
         </is>
       </c>
-      <c r="C11" s="29" t="n"/>
-      <c r="D11" s="29" t="n"/>
-      <c r="E11" s="29" t="n"/>
-      <c r="F11" s="29" t="n"/>
     </row>
     <row r="12" ht="16" customHeight="1">
       <c r="B12" s="39" t="inlineStr">
@@ -843,10 +835,10 @@
           <t>1. Keywords analíticas en is_pdf_content_query (rag_retriever.php, línea 1622)</t>
         </is>
       </c>
-      <c r="C12" s="40" t="n"/>
-      <c r="D12" s="40" t="n"/>
-      <c r="E12" s="40" t="n"/>
-      <c r="F12" s="40" t="n"/>
+      <c r="C12" s="17" t="n"/>
+      <c r="D12" s="17" t="n"/>
+      <c r="E12" s="17" t="n"/>
+      <c r="F12" s="20" t="n"/>
     </row>
     <row r="13" ht="46" customHeight="1">
       <c r="B13" s="41" t="inlineStr">
@@ -854,10 +846,10 @@
           <t>EL MÁS GRAVE. Rompe el caso de uso central (notas, matriculados): esas preguntas se enrutan a 'modo documento' y responden 'el documento no proporciona información'. Afecta: P12, P15, P16, P25, P28, P29, P45, P52.  Fix: una línea.</t>
         </is>
       </c>
-      <c r="C13" s="40" t="n"/>
-      <c r="D13" s="40" t="n"/>
-      <c r="E13" s="40" t="n"/>
-      <c r="F13" s="40" t="n"/>
+      <c r="C13" s="17" t="n"/>
+      <c r="D13" s="17" t="n"/>
+      <c r="E13" s="17" t="n"/>
+      <c r="F13" s="20" t="n"/>
     </row>
     <row r="14" ht="16" customHeight="1">
       <c r="B14" s="39" t="inlineStr">
@@ -865,10 +857,10 @@
           <t>2. El matcher engancha por palabra genérica ('alumno', 'nota', 'resumen')</t>
         </is>
       </c>
-      <c r="C14" s="40" t="n"/>
-      <c r="D14" s="40" t="n"/>
-      <c r="E14" s="40" t="n"/>
-      <c r="F14" s="40" t="n"/>
+      <c r="C14" s="17" t="n"/>
+      <c r="D14" s="17" t="n"/>
+      <c r="E14" s="17" t="n"/>
+      <c r="F14" s="20" t="n"/>
     </row>
     <row r="15" ht="46" customHeight="1">
       <c r="B15" s="41" t="inlineStr">
@@ -876,10 +868,10 @@
           <t>PRIORIDAD ALTA. Devuelve un PDF cualquiera que comparta una palabra con la pregunta; rompe incluso los botones (P33) y los seguimientos conversacionales. Afecta: P4, P6, P30, P31, P32, P34, P39, P53, P54, P33.</t>
         </is>
       </c>
-      <c r="C15" s="40" t="n"/>
-      <c r="D15" s="40" t="n"/>
-      <c r="E15" s="40" t="n"/>
-      <c r="F15" s="40" t="n"/>
+      <c r="C15" s="17" t="n"/>
+      <c r="D15" s="17" t="n"/>
+      <c r="E15" s="17" t="n"/>
+      <c r="F15" s="20" t="n"/>
     </row>
     <row r="16" ht="16" customHeight="1">
       <c r="B16" s="42" t="inlineStr">
@@ -887,10 +879,10 @@
           <t>3. Contaminación de contexto / history-hint</t>
         </is>
       </c>
-      <c r="C16" s="43" t="n"/>
-      <c r="D16" s="43" t="n"/>
-      <c r="E16" s="43" t="n"/>
-      <c r="F16" s="43" t="n"/>
+      <c r="C16" s="17" t="n"/>
+      <c r="D16" s="17" t="n"/>
+      <c r="E16" s="17" t="n"/>
+      <c r="F16" s="20" t="n"/>
     </row>
     <row r="17" ht="46" customHeight="1">
       <c r="B17" s="44" t="inlineStr">
@@ -898,10 +890,10 @@
           <t>Reproducido: con el chat sucio arrastra recursos de turnos anteriores; Ctrl+F5 lo arregla. Afecta: P14, P37, P38, P50, P51.</t>
         </is>
       </c>
-      <c r="C17" s="43" t="n"/>
-      <c r="D17" s="43" t="n"/>
-      <c r="E17" s="43" t="n"/>
-      <c r="F17" s="43" t="n"/>
+      <c r="C17" s="17" t="n"/>
+      <c r="D17" s="17" t="n"/>
+      <c r="E17" s="17" t="n"/>
+      <c r="F17" s="20" t="n"/>
     </row>
     <row r="18" ht="16" customHeight="1">
       <c r="B18" s="42" t="inlineStr">
@@ -909,10 +901,10 @@
           <t>4. Extracción de PDF rota</t>
         </is>
       </c>
-      <c r="C18" s="43" t="n"/>
-      <c r="D18" s="43" t="n"/>
-      <c r="E18" s="43" t="n"/>
-      <c r="F18" s="43" t="n"/>
+      <c r="C18" s="17" t="n"/>
+      <c r="D18" s="17" t="n"/>
+      <c r="E18" s="17" t="n"/>
+      <c r="F18" s="20" t="n"/>
     </row>
     <row r="19" ht="46" customHeight="1">
       <c r="B19" s="44" t="inlineStr">
@@ -920,10 +912,10 @@
           <t>Confirmado en sandbox: pdftotext SÍ extrae el texto; el parser del plugin no (fuentes CID/Identity-H). No hace falta OCR. Afecta: P22, P23, P24.  Fix: instalar poppler-utils / smalot.</t>
         </is>
       </c>
-      <c r="C19" s="43" t="n"/>
-      <c r="D19" s="43" t="n"/>
-      <c r="E19" s="43" t="n"/>
-      <c r="F19" s="43" t="n"/>
+      <c r="C19" s="17" t="n"/>
+      <c r="D19" s="17" t="n"/>
+      <c r="E19" s="17" t="n"/>
+      <c r="F19" s="20" t="n"/>
     </row>
     <row r="20" ht="16" customHeight="1">
       <c r="B20" s="42" t="inlineStr">
@@ -931,10 +923,10 @@
           <t>5. Referencias por posición ('el primero/segundo') no se resuelven</t>
         </is>
       </c>
-      <c r="C20" s="43" t="n"/>
-      <c r="D20" s="43" t="n"/>
-      <c r="E20" s="43" t="n"/>
-      <c r="F20" s="43" t="n"/>
+      <c r="C20" s="17" t="n"/>
+      <c r="D20" s="17" t="n"/>
+      <c r="E20" s="17" t="n"/>
+      <c r="F20" s="20" t="n"/>
     </row>
     <row r="21" ht="46" customHeight="1">
       <c r="B21" s="44" t="inlineStr">
@@ -942,10 +934,10 @@
           <t>Las interpreta por keyword y engancha una actividad equivocada. Afecta: P51.</t>
         </is>
       </c>
-      <c r="C21" s="43" t="n"/>
-      <c r="D21" s="43" t="n"/>
-      <c r="E21" s="43" t="n"/>
-      <c r="F21" s="43" t="n"/>
+      <c r="C21" s="17" t="n"/>
+      <c r="D21" s="17" t="n"/>
+      <c r="E21" s="17" t="n"/>
+      <c r="F21" s="20" t="n"/>
     </row>
     <row r="22" ht="16" customHeight="1">
       <c r="B22" s="45" t="inlineStr">
@@ -953,10 +945,10 @@
           <t>6. Huecos de funcionalidad</t>
         </is>
       </c>
-      <c r="C22" s="46" t="n"/>
-      <c r="D22" s="46" t="n"/>
-      <c r="E22" s="46" t="n"/>
-      <c r="F22" s="46" t="n"/>
+      <c r="C22" s="17" t="n"/>
+      <c r="D22" s="17" t="n"/>
+      <c r="E22" s="17" t="n"/>
+      <c r="F22" s="20" t="n"/>
     </row>
     <row r="23" ht="46" customHeight="1">
       <c r="B23" s="47" t="inlineStr">
@@ -964,10 +956,10 @@
           <t>Contenido Office .docx/.pptx (P39), ranking de alumnos (P34), contenido de SCORM (P55/P56 — justo lo que hace Phia).</t>
         </is>
       </c>
-      <c r="C23" s="46" t="n"/>
-      <c r="D23" s="46" t="n"/>
-      <c r="E23" s="46" t="n"/>
-      <c r="F23" s="46" t="n"/>
+      <c r="C23" s="17" t="n"/>
+      <c r="D23" s="17" t="n"/>
+      <c r="E23" s="17" t="n"/>
+      <c r="F23" s="20" t="n"/>
     </row>
     <row r="25" ht="24" customHeight="1">
       <c r="B25" s="28" t="inlineStr">
@@ -975,10 +967,6 @@
           <t>Lo que funciona bien</t>
         </is>
       </c>
-      <c r="C25" s="29" t="n"/>
-      <c r="D25" s="29" t="n"/>
-      <c r="E25" s="29" t="n"/>
-      <c r="F25" s="29" t="n"/>
     </row>
     <row r="26" ht="46" customHeight="1">
       <c r="B26" s="48" t="inlineStr">
@@ -993,10 +981,6 @@
           <t>Recomendación de orden de arreglo</t>
         </is>
       </c>
-      <c r="C28" s="29" t="n"/>
-      <c r="D28" s="29" t="n"/>
-      <c r="E28" s="29" t="n"/>
-      <c r="F28" s="29" t="n"/>
     </row>
     <row r="29" ht="46" customHeight="1">
       <c r="B29" s="38" t="inlineStr">
@@ -1771,7 +1755,7 @@
           <t>Bien</t>
         </is>
       </c>
-      <c r="E14" s="14" t="inlineStr">
+      <c r="E14" s="13" t="inlineStr">
         <is>
           <t>Bien</t>
         </is>
@@ -1783,7 +1767,7 @@
       </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
-          <t>Correcto, ruta directa. El curso sí tiene un quiz real ('Cuestionario tipo test').</t>
+          <t>[✓ RECUPERADA con fix #2 (v1.1.4): 'tiene 15 preguntas'. El match exacto del quiz gana; ya no lo secuestra un PDF.]  Correcto, ruta directa. El curso sí tiene un quiz real ('Cuestionario tipo test'). [OJO: tras el fix #1, en cursos con un recurso cuyo nombre contiene 'tipo'/'test'/'cuestionario', esta pregunta la intercepta el bug #2 (el matcher agarra el recurso antes que el quiz) y falla con 'no aparece en el documento'. NO es regresion del fix #1 (commit solo toco la regex + version; la logica de conteo esta intacta). Se recupera con el fix #2.]</t>
         </is>
       </c>
       <c r="H14" s="21" t="n"/>
@@ -1859,7 +1843,7 @@
       </c>
       <c r="G16" s="14" t="inlineStr">
         <is>
-          <t>BUG. La frase 'el documento no proporciona informacion' es del modo documento (answer_document_question), no de la rama de nota. O bien no disparo $asksGradeData en build_quiz_answer, o el calculo de media (sumgrades) devolvio null/0 y cayo a una respuesta de documento enganosa. Contradice P10/P11 que si funcionaron por ruta directa sobre el mismo quiz. [CAUSA RAIZ CONFIRMADA EN CODIGO: rag_retriever.php linea 1622, is_pdf_content_query incluye 'nota media|calificacion media/promedio|cuantos alumnos/estudiantes|quien ha completado|cuantos intentos'. Por eso estas preguntas se clasifican como 'contenido de documento' (isContentIntent=true) y se responden sobre un PDF -&gt; 'el documento no menciona'. Verificado tambien en curso CON notas: 'nota media del curso' falla igual mientras '% aprobados' funciona.]</t>
+          <t>[PROBABLEMENTE RECUPERADA tras fix #1+#2 (v1.1.4), misma raiz que P25/P30 — PENDIENTE de confirmar en chat.]  BUG. La frase 'el documento no proporciona informacion' es del modo documento (answer_document_question), no de la rama de nota. O bien no disparo $asksGradeData en build_quiz_answer, o el calculo de media (sumgrades) devolvio null/0 y cayo a una respuesta de documento enganosa. Contradice P10/P11 que si funcionaron por ruta directa sobre el mismo quiz. [CAUSA RAIZ CONFIRMADA EN CODIGO: rag_retriever.php linea 1622, is_pdf_content_query incluye 'nota media|calificacion media/promedio|cuantos alumnos/estudiantes|quien ha completado|cuantos intentos'. Por eso estas preguntas se clasifican como 'contenido de documento' (isContentIntent=true) y se responden sobre un PDF -&gt; 'el documento no menciona'. Verificado tambien en curso CON notas: 'nota media del curso' falla igual mientras '% aprobados' funciona.]</t>
         </is>
       </c>
       <c r="H16" s="21" t="inlineStr">
@@ -1986,7 +1970,7 @@
       </c>
       <c r="G19" s="14" t="inlineStr">
         <is>
-          <t>MISMO BUG que P12 (nota media), aqui en tarea. Las consultas de 'nota media' caen al modo documento (answer_document_question) y devuelven 'no se menciona en el documento' en vez de calcular la media desde assign_grades. Nota positiva: el matching de la tarea SI funciono aqui, lo que confirma que el fallo de P14 fue contaminacion del history-hint. [CAUSA RAIZ CONFIRMADA EN CODIGO: rag_retriever.php linea 1622, is_pdf_content_query incluye 'nota media|calificacion media/promedio|cuantos alumnos/estudiantes|quien ha completado|cuantos intentos'. Por eso estas preguntas se clasifican como 'contenido de documento' (isContentIntent=true) y se responden sobre un PDF -&gt; 'el documento no menciona'. Verificado tambien en curso CON notas: 'nota media del curso' falla igual mientras '% aprobados' funciona.]</t>
+          <t>[PROBABLEMENTE RECUPERADA tras fix #1+#2 (v1.1.4), misma raiz que P25/P30 — PENDIENTE de confirmar en chat.]  MISMO BUG que P12 (nota media), aqui en tarea. Las consultas de 'nota media' caen al modo documento (answer_document_question) y devuelven 'no se menciona en el documento' en vez de calcular la media desde assign_grades. Nota positiva: el matching de la tarea SI funciono aqui, lo que confirma que el fallo de P14 fue contaminacion del history-hint. [CAUSA RAIZ CONFIRMADA EN CODIGO: rag_retriever.php linea 1622, is_pdf_content_query incluye 'nota media|calificacion media/promedio|cuantos alumnos/estudiantes|quien ha completado|cuantos intentos'. Por eso estas preguntas se clasifican como 'contenido de documento' (isContentIntent=true) y se responden sobre un PDF -&gt; 'el documento no menciona'. Verificado tambien en curso CON notas: 'nota media del curso' falla igual mientras '% aprobados' funciona.]</t>
         </is>
       </c>
       <c r="H19" s="21" t="inlineStr">
@@ -2016,9 +2000,9 @@
           <t>Bien</t>
         </is>
       </c>
-      <c r="E20" s="14" t="inlineStr">
-        <is>
-          <t>Mal</t>
+      <c r="E20" s="13" t="inlineStr">
+        <is>
+          <t>Bien</t>
         </is>
       </c>
       <c r="F20" s="19" t="inlineStr">
@@ -2028,7 +2012,7 @@
       </c>
       <c r="G20" s="14" t="inlineStr">
         <is>
-          <t>BUG importante y de caso de uso central ('cuantos alumnos hay'). El dato existe: count_enrolled_users() y el total en el contexto analitico (metadata total_enrolled). Pero la consulta se enruta a RAG/documento y el modelo responde que no esta en el documento. Probable causa doble: (1) no hay ruta directa para 'cuantos alumnos matriculados'; (2) el system prompt 'REGLA CRITICA DE CONSISTENCIA' hace que el modelo solo mire los fragmentos RAG e ignore el JSON de analitica, o el JSON no se esta inyectando. [CAUSA RAIZ CONFIRMADA EN CODIGO: rag_retriever.php linea 1622, is_pdf_content_query incluye 'nota media|calificacion media/promedio|cuantos alumnos/estudiantes|quien ha completado|cuantos intentos'. Por eso estas preguntas se clasifican como 'contenido de documento' (isContentIntent=true) y se responden sobre un PDF -&gt; 'el documento no menciona'. Verificado tambien en curso CON notas: 'nota media del curso' falla igual mientras '% aprobados' funciona.]</t>
+          <t>[✓ RECUPERADA con fix #1+#2 (v1.1.4): 'Hay un total de 13 estudiantes matriculados' + tabla + export. Va por analitica.]  BUG importante y de caso de uso central ('cuantos alumnos hay'). El dato existe: count_enrolled_users() y el total en el contexto analitico (metadata total_enrolled). Pero la consulta se enruta a RAG/documento y el modelo responde que no esta en el documento. Probable causa doble: (1) no hay ruta directa para 'cuantos alumnos matriculados'; (2) el system prompt 'REGLA CRITICA DE CONSISTENCIA' hace que el modelo solo mire los fragmentos RAG e ignore el JSON de analitica, o el JSON no se esta inyectando. [CAUSA RAIZ CONFIRMADA EN CODIGO: rag_retriever.php linea 1622, is_pdf_content_query incluye 'nota media|calificacion media/promedio|cuantos alumnos/estudiantes|quien ha completado|cuantos intentos'. Por eso estas preguntas se clasifican como 'contenido de documento' (isContentIntent=true) y se responden sobre un PDF -&gt; 'el documento no menciona'. Verificado tambien en curso CON notas: 'nota media del curso' falla igual mientras '% aprobados' funciona.]</t>
         </is>
       </c>
       <c r="H20" s="21" t="inlineStr">
@@ -2441,9 +2425,9 @@
           <t>Mal</t>
         </is>
       </c>
-      <c r="E32" s="14" t="inlineStr">
-        <is>
-          <t>Mal</t>
+      <c r="E32" s="13" t="inlineStr">
+        <is>
+          <t>Bien</t>
         </is>
       </c>
       <c r="F32" s="19" t="inlineStr">
@@ -2453,7 +2437,7 @@
       </c>
       <c r="G32" s="14" t="inlineStr">
         <is>
-          <t>Confirmado el patron de P12/P15/P16: las preguntas de analitica caen a modo documento. Ademas data_retriever NO agrega (no calcula media de curso), y el saludo del bot promete 'preguntame sobre notas/completitud/estudiantes en riesgo' -&gt; choque de expectativas grave: promete analitica y falla en la analitica basica. [CAUSA RAIZ CONFIRMADA EN CODIGO: rag_retriever.php linea 1622, is_pdf_content_query incluye 'nota media|calificacion media/promedio|cuantos alumnos/estudiantes|quien ha completado|cuantos intentos'. Por eso estas preguntas se clasifican como 'contenido de documento' (isContentIntent=true) y se responden sobre un PDF -&gt; 'el documento no menciona'. Verificado tambien en curso CON notas: 'nota media del curso' falla igual mientras '% aprobados' funciona.]</t>
+          <t>[✓ RECUPERADA con fix #1+#2 (v1.1.4): 'La calificacion media es 8.53 sobre 10' (con contexto limpio). Ya no dice 'el documento no proporciona'.]  Confirmado el patron de P12/P15/P16: las preguntas de analitica caen a modo documento. Ademas data_retriever NO agrega (no calcula media de curso), y el saludo del bot promete 'preguntame sobre notas/completitud/estudiantes en riesgo' -&gt; choque de expectativas grave: promete analitica y falla en la analitica basica. [CAUSA RAIZ CONFIRMADA EN CODIGO: rag_retriever.php linea 1622, is_pdf_content_query incluye 'nota media|calificacion media/promedio|cuantos alumnos/estudiantes|quien ha completado|cuantos intentos'. Por eso estas preguntas se clasifican como 'contenido de documento' (isContentIntent=true) y se responden sobre un PDF -&gt; 'el documento no menciona'. Verificado tambien en curso CON notas: 'nota media del curso' falla igual mientras '% aprobados' funciona.]</t>
         </is>
       </c>
       <c r="H32" s="21" t="inlineStr">
@@ -2586,7 +2570,7 @@
       </c>
       <c r="G35" s="14" t="inlineStr">
         <is>
-          <t>MISMO bug de la linea 1622 (is_pdf_content_query captura 'nota media'). Confirma que cualquier fraseo con 'nota media' falla. Ver P25 para causa raiz y fix.</t>
+          <t>[PROBABLEMENTE RECUPERADA tras fix #1+#2 (v1.1.4), misma raiz que P25/P30 — PENDIENTE de confirmar en chat.]  MISMO bug de la linea 1622 (is_pdf_content_query captura 'nota media'). Confirma que cualquier fraseo con 'nota media' falla. Ver P25 para causa raiz y fix.</t>
         </is>
       </c>
       <c r="H35" s="21" t="inlineStr">
@@ -2628,7 +2612,7 @@
       </c>
       <c r="G36" s="14" t="inlineStr">
         <is>
-          <t>MISMA raiz linea 1622: 'cuantos alumnos' esta en is_pdf_content_query -&gt; isContentIntent=true -&gt; busca un recurso/actividad y engancha el foro que contiene 'alumnos' en su nombre (fallo de matching combinado). El dato de finalizacion del curso existe (get_course_completions). Doble bug: enrutado (1622) + matching por nombre.</t>
+          <t>[PROBABLEMENTE RECUPERADA tras fix #1+#2 (v1.1.4), misma raiz que P25/P30 — PENDIENTE de confirmar en chat.]  MISMA raiz linea 1622: 'cuantos alumnos' esta en is_pdf_content_query -&gt; isContentIntent=true -&gt; busca un recurso/actividad y engancha el foro que contiene 'alumnos' en su nombre (fallo de matching combinado). El dato de finalizacion del curso existe (get_course_completions). Doble bug: enrutado (1622) + matching por nombre.</t>
         </is>
       </c>
       <c r="H36" s="21" t="inlineStr">
@@ -2679,9 +2663,9 @@
           <t>Mal</t>
         </is>
       </c>
-      <c r="E38" s="14" t="inlineStr">
-        <is>
-          <t>Mal</t>
+      <c r="E38" s="13" t="inlineStr">
+        <is>
+          <t>Bien</t>
         </is>
       </c>
       <c r="F38" s="19" t="inlineStr">
@@ -2691,17 +2675,23 @@
       </c>
       <c r="G38" s="14" t="inlineStr">
         <is>
-          <t>Doble problema: (1) HUECO DE FUNCIONALIDAD: no existe ranking de alumnos por nota. (2) BUG matching: en vez de responder 'no puedo dar rankings', el matcher agarra cualquier recurso que comparta una palabra generica ('alumno'/'nota') con la pregunta. Misma familia que P4/P6/P14/P29.</t>
+          <t>[✓ RECUPERADA con fix #2 (v1.1.4): da ranking real (mejor nota: Maria Petra Gordillo, 10/10) con insights, en vez de enganchar 'Guia del alumno'. NOTA: expone nombre+email del alumno -&gt; revisar privacidad (P32).]  Doble problema: (1) HUECO DE FUNCIONALIDAD: no existe ranking de alumnos por nota. (2) BUG matching: en vez de responder 'no puedo dar rankings', el matcher agarra cualquier recurso que comparta una palabra generica ('alumno'/'nota') con la pregunta. Misma familia que P4/P6/P14/P29.</t>
         </is>
       </c>
       <c r="H38" s="21" t="inlineStr">
         <is>
-          <t>Contexto: Plugin de Moodle `block_pulso`. Fichero: classes/rag_retriever.php, funcion `match_activity_by_name()`. IMPORTANTE: este bug es de ALTA PRIORIDAD porque afecta tambien a las funciones accesibles por boton (En riesgo, Notas, etc.), no solo a preguntas escritas.
-Sintoma: Preguntas de analitica sobre alumnos ('¿quien es el alumno con mejor nota?', '¿que alumnos van peor?', '¿que estudiantes estan en riesgo?') devuelven los METADATOS de un recurso PDF cuyo nombre contiene una palabra generica de la pregunta: 'Guia del alumno' (por 'alumno'), 'NOTA INFORMATIVA...' (por 'nota'), 'Manual... del estudiante' (por 'estudiante'). Incluso el boton 'En riesgo' falla en cursos que tienen un PDF con esas palabras en el nombre.
-Causa raiz: `match_activity_by_name()` empareja una actividad/recurso cuando comparte UNA sola palabra generica con la pregunta, y devuelve ese recurso al azar en vez de reconocer que es una intencion analitica.
-Arreglo: (1) Sube el umbral de coincidencia: no emparejar por una sola palabra generica. Anade a stopwords palabras como 'alumno','alumnos','estudiante','estudiantes','nota','notas','participante','participantes','guia','manual', o exige coincidencia de la mayor parte del nombre. (2) Si no hay match claro, NO devuelvas un recurso: deja que la consulta siga hacia la ruta analitica/LLM. (3) Da PRIORIDAD a las intenciones analiticas (en riesgo, notas, completitud, engagement, ranking) sobre el match de actividad en `resolve_direct_course_query()`.
-No romper: cuando el usuario nombra un recurso de forma inequivoca, el match debe seguir funcionando.
-VERSIONADO (OBLIGATORIO, regla del proyecto): sube tanto $plugin-&gt;version (formato YYYYMMDDXX) como $plugin-&gt;release (semver) en version.php. Aplica en cada cambio, por pequeno que sea.</t>
+          <t>BUG #2 — El matcher engancha un recurso por palabra generica y se salta el quiz/tarea/analitica.
+Contexto: Plugin de Moodle block_pulso. Fichero: classes/rag_retriever.php, funciones resolve_direct_resource_query() (~linea 309) y match_activity_by_name() (~lineas 521-563). ALTA PRIORIDAD: afecta preguntas escritas, seguimientos conversacionales y hasta los botones (En riesgo/Notas).
+Sintoma: preguntas de analitica o sobre una actividad concreta devuelven los METADATOS de un PDF cuyo nombre comparte una palabra con la pregunta: 'nota media' -&gt; engancha 'NOTA INFORMATIVA'; 'cuantos alumnos' -&gt; 'Foro de presentacion de alumnos'; 'quien es el alumno con mejor nota' -&gt; 'Guia del alumno'; y hasta 'cuantas preguntas tiene el cuestionario tipo test' -&gt; un PDF con 'tipo'/'test'/'cuestionario' en el nombre, en vez de responder con el quiz.
+Causa raiz (confirmada por trazado):
+(1) En resolve_direct_resource_query() se intenta emparejar un RECURSO PRIMERO (linea 345) y solo si no hay match se prueba quiz (350), assign (358), etc. Asi, un recurso con un token generico gana antes de llegar al quiz/tarea.
+(2) match_activity_by_name() (~544-559) puntua cualquier palabra de &gt;=4 letras; palabras genericas como 'tipo','test','curso','nota','alumno','estudiante','foro','tarea','resumen','cuestionario' SI puntuan, y con una sola coincidencia ya devuelve ese recurso.
+Arreglo:
+(A) match_activity_by_name(): subir el umbral. No emparejar por una sola palabra generica; puntuar sobre el nombre COMPLETO; ampliar la stopword-list con 'tipo','test','curso','nota','notas','alumno','alumnos','estudiante','estudiantes','foro','tarea','resumen','participante','participantes','guia','manual','cuestionario','actividad','pregunta','preguntas'; usar numeros/ordinales como discriminador; si no hay match claro, devolver null (que la consulta siga a analitica/LLM).
+(B) Enrutado: no dar por defecto prioridad al recurso. Si la pregunta contiene una pista de TIPO de actividad ('cuestionario'-&gt;quiz, 'tarea'-&gt;assign, 'foro'-&gt;forum), probar ese tipo ANTES que los recursos. Alternativa mejor: puntuar candidatos de TODOS los tipos y quedarse con el de mayor score, no 'recurso primero'.
+(C) Prioridad de intenciones analiticas: si la pregunta es de analitica (nota media, matriculados, en riesgo, completitud, ranking), esa ruta debe ir ANTES del match de actividad/recurso.
+No romper: cuando el usuario nombra un recurso de forma inequivoca (nombre completo y distintivo), el match debe seguir funcionando. Verifica que P10 ('cuantas preguntas tiene el cuestionario tipo test') vuelve a dar el numero de preguntas, que 'nota media del curso' y 'cuantos alumnos matriculados' van a analitica, y que 'que contiene el recurso X' (nombre claro) sigue resolviendo el PDF correcto.
+VERSIONADO (OBLIGATORIO): sube $plugin-&gt;version (YYYYMMDDXX) y $plugin-&gt;release (semver) en version.php.</t>
         </is>
       </c>
       <c r="I38" s="22" t="n"/>
@@ -3362,7 +3352,7 @@
       </c>
       <c r="G56" s="14" t="inlineStr">
         <is>
-          <t>Fraseo coloquial de nota media. Combina los dos bugs habituales: (1) 'nota...media' captura la intencion de contenido (linea 1622); (2) el matcher engancha 'NOTA INFORMATIVA' por la palabra 'nota'. Distinto de P28 (que dio texto): aqui saco un recurso.</t>
+          <t>[PROBABLEMENTE RECUPERADA tras fix #1+#2 (v1.1.4), misma raiz que P25/P30 — PENDIENTE de confirmar en chat.]  Fraseo coloquial de nota media. Combina los dos bugs habituales: (1) 'nota...media' captura la intencion de contenido (linea 1622); (2) el matcher engancha 'NOTA INFORMATIVA' por la palabra 'nota'. Distinto de P28 (que dio texto): aqui saco un recurso.</t>
         </is>
       </c>
       <c r="H56" s="21" t="inlineStr">

</xml_diff>

<commit_message>
Actualiza matriz: re-verificacion con Claude y fixes 6.x
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Pulso_AI_matriz_evaluacion.xlsx
+++ b/Pulso_AI_matriz_evaluacion.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30309"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30305"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_EB5570BF012881FB0A7950BAFCD4C2FE933BBE55" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{95CD2AA2-C519-4222-B59D-C92876E44E78}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_EB5570BF012881FB0A89DC739C34FD32933B86F0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -472,7 +472,7 @@
     <t>Dos variantes ('cuantos alumnos hay matriculados' y '...en este curso'), ambas: 'El documento no especifica / no aparece en el documento proporcionado el numero de alumnos matriculados'. No dio el numero.</t>
   </si>
   <si>
-    <t>[✓ RECUPERADA con fix #1+#2 (v1.1.4): 'Hay un total de 13 estudiantes matriculados' + tabla + export. Va por analitica.]  BUG importante y de caso de uso central ('cuantos alumnos hay'). El dato existe: count_enrolled_users() y el total en el contexto analitico (metadata total_enrolled). Pero la consulta se enruta a RAG/documento y el modelo responde que no esta en el documento. Probable causa doble: (1) no hay ruta directa para 'cuantos alumnos matriculados'; (2) el system prompt 'REGLA CRITICA DE CONSISTENCIA' hace que el modelo solo mire los fragmentos RAG e ignore el JSON de analitica, o el JSON no se esta inyectando. [CAUSA RAIZ CONFIRMADA EN CODIGO: rag_retriever.php linea 1622, is_pdf_content_query incluye 'nota media|calificacion media/promedio|cuantos alumnos/estudiantes|quien ha completado|cuantos intentos'. Por eso estas preguntas se clasifican como 'contenido de documento' (isContentIntent=true) y se responden sobre un PDF -&gt; 'el documento no menciona'. Verificado tambien en curso CON notas: 'nota media del curso' falla igual mientras '% aprobados' funciona.]</t>
+    <t>[✓✓ RE-VERIFICADA con Claude (v1.2.4): 15 totales / 13 alumnos / 2 staff + tabla + export. Mas matizada que con gpt-4o.]  [✓ RECUPERADA con fix #1+#2 (v1.1.4): 'Hay un total de 13 estudiantes matriculados' + tabla + export. Va por analitica.]  BUG importante y de caso de uso central ('cuantos alumnos hay'). El dato existe: count_enrolled_users() y el total en el contexto analitico (metadata total_enrolled). Pero la consulta se enruta a RAG/documento y el modelo responde que no esta en el documento. Probable causa doble: (1) no hay ruta directa para 'cuantos alumnos matriculados'; (2) el system prompt 'REGLA CRITICA DE CONSISTENCIA' hace que el modelo solo mire los fragmentos RAG e ignore el JSON de analitica, o el JSON no se esta inyectando. [CAUSA RAIZ CONFIRMADA EN CODIGO: rag_retriever.php linea 1622, is_pdf_content_query incluye 'nota media|calificacion media/promedio|cuantos alumnos/estudiantes|quien ha completado|cuantos intentos'. Por eso estas preguntas se clasifican como 'contenido de documento' (isContentIntent=true) y se responden sobre un PDF -&gt; 'el documento no menciona'. Verificado tambien en curso CON notas: 'nota media del curso' falla igual mientras '% aprobados' funciona.]</t>
   </si>
   <si>
     <t>Contexto: Plugin de Moodle `block_pulso`. Ficheros: classes/rag_retriever.php, classes/data_retriever.php, classes/system_prompt_designer.php.
@@ -606,7 +606,7 @@
     <t>'El documento no proporciona informacion sobre la nota media del curso.' No calculo la media global.</t>
   </si>
   <si>
-    <t>[✓ RECUPERADA con fix #1+#2 (v1.1.4): 'La calificacion media es 8.53 sobre 10' (con contexto limpio). Ya no dice 'el documento no proporciona'.]  Confirmado el patron de P12/P15/P16: las preguntas de analitica caen a modo documento. Ademas data_retriever NO agrega (no calcula media de curso), y el saludo del bot promete 'preguntame sobre notas/completitud/estudiantes en riesgo' -&gt; choque de expectativas grave: promete analitica y falla en la analitica basica. [CAUSA RAIZ CONFIRMADA EN CODIGO: rag_retriever.php linea 1622, is_pdf_content_query incluye 'nota media|calificacion media/promedio|cuantos alumnos/estudiantes|quien ha completado|cuantos intentos'. Por eso estas preguntas se clasifican como 'contenido de documento' (isContentIntent=true) y se responden sobre un PDF -&gt; 'el documento no menciona'. Verificado tambien en curso CON notas: 'nota media del curso' falla igual mientras '% aprobados' funciona.]</t>
+    <t>[✓✓ RE-VERIFICADA con Claude Sonnet 5 (v1.2.4): '9.18/10 (91.85%)' + tabla con badges; distingue 9 de 13 y excluye staff. Renderiza bien. Calidad mejorada vs gpt-4o.]  [✓ RECUPERADA con fix #1+#2 (v1.1.4): 'La calificacion media es 8.53 sobre 10' (con contexto limpio). Ya no dice 'el documento no proporciona'.]  Confirmado el patron de P12/P15/P16: las preguntas de analitica caen a modo documento. Ademas data_retriever NO agrega (no calcula media de curso), y el saludo del bot promete 'preguntame sobre notas/completitud/estudiantes en riesgo' -&gt; choque de expectativas grave: promete analitica y falla en la analitica basica. [CAUSA RAIZ CONFIRMADA EN CODIGO: rag_retriever.php linea 1622, is_pdf_content_query incluye 'nota media|calificacion media/promedio|cuantos alumnos/estudiantes|quien ha completado|cuantos intentos'. Por eso estas preguntas se clasifican como 'contenido de documento' (isContentIntent=true) y se responden sobre un PDF -&gt; 'el documento no menciona'. Verificado tambien en curso CON notas: 'nota media del curso' falla igual mientras '% aprobados' funciona.]</t>
   </si>
   <si>
     <t>Contexto: Plugin de Moodle `block_pulso` (chat de analitica con IA sobre cursos). Tiene una ruta de analitica (responde con notas, insights, etc.) y una ruta de contenido de documento. Fichero: classes/rag_retriever.php.
@@ -627,7 +627,7 @@
     <t>Respuesta estructurada (formato analitica: Insights + Recomendaciones). Dijo que no hay calificaciones/aprobados registrados en ADGD0208, con recomendaciones (revisar config de calificaciones, asegurar que los alumnos completen evaluaciones). Sin alucinar.</t>
   </si>
   <si>
-    <t>MUY REVELADOR. Aqui SI uso la ruta de analitica (formato con insights/recomendaciones), a diferencia de P25 (misma tematica de notas) que cayo a modo documento. CONCLUSION CLAVE: la ruta de analitica funciona bien; el bug de P12/P15/P16/P25 es ENRUTADO INCOHERENTE (unas preguntas de notas van a analitica y otras a modo documento). A VERIFICAR: dice 'no hay notas' pero el quiz tenia 10 intentos finalizados (P11); revisar si las notas del quiz llegan al gradebook (grades_and_quizzes). [EVIDENCIA EXTRA: la misma pregunta en OTRO curso CON notas da respuesta excelente: tabla (9 completaron / 9 aprobados / 100%), insights, recomendaciones y export Excel/CSV. Confirma que la ruta de analitica calcula bien % aprobados cuando hay datos. El bug de P12/P15/P25 es de ENRUTADO de la consulta 'nota media' a modo documento, no de capacidad analitica.]</t>
+    <t>[✓✓ RE-VERIFICADA con Claude (v1.2.4): distingue % sobre presentados vs total + insights.]  MUY REVELADOR. Aqui SI uso la ruta de analitica (formato con insights/recomendaciones), a diferencia de P25 (misma tematica de notas) que cayo a modo documento. CONCLUSION CLAVE: la ruta de analitica funciona bien; el bug de P12/P15/P16/P25 es ENRUTADO INCOHERENTE (unas preguntas de notas van a analitica y otras a modo documento). A VERIFICAR: dice 'no hay notas' pero el quiz tenia 10 intentos finalizados (P11); revisar si las notas del quiz llegan al gradebook (grades_and_quizzes). [EVIDENCIA EXTRA: la misma pregunta en OTRO curso CON notas da respuesta excelente: tabla (9 completaron / 9 aprobados / 100%), insights, recomendaciones y export Excel/CSV. Confirma que la ruta de analitica calcula bien % aprobados cuando hay datos. El bug de P12/P15/P25 es de ENRUTADO de la consulta 'nota media' a modo documento, no de capacidad analitica.]</t>
   </si>
   <si>
     <t>¿Qué porcentaje de actividades se han completado de media?</t>
@@ -697,7 +697,7 @@
     <t>En 2 cursos distintos, ambos mal: (1) engancho el recurso 'Guia del alumno' (GA_ADGD0208...pdf) por el token 'alumno'; (2) engancho 'NOTA INFORMATIVA DIRIGIDA A LOS PARTICIPANTES' por el token 'nota'. Devolvio metadatos de un PDF, no un ranking.</t>
   </si>
   <si>
-    <t>[✓ RECUPERADA con fix #2 (v1.1.4): da ranking real (mejor nota: Maria Petra Gordillo, 10/10) con insights, en vez de enganchar 'Guia del alumno'. NOTA: expone nombre+email del alumno -&gt; revisar privacidad (P32).]  Doble problema: (1) HUECO DE FUNCIONALIDAD: no existe ranking de alumnos por nota. (2) BUG matching: en vez de responder 'no puedo dar rankings', el matcher agarra cualquier recurso que comparta una palabra generica ('alumno'/'nota') con la pregunta. Misma familia que P4/P6/P14/P29.</t>
+    <t>[✓✓ RE-VERIFICADA con Claude (v1.2.4): ranking/mejor alumno renderiza bien, sin email.]  [✓ RECUPERADA con fix #2 (v1.1.4): da ranking real (mejor nota: Maria Petra Gordillo, 10/10) con insights, en vez de enganchar 'Guia del alumno'. NOTA: expone nombre+email del alumno -&gt; revisar privacidad (P32).]  Doble problema: (1) HUECO DE FUNCIONALIDAD: no existe ranking de alumnos por nota. (2) BUG matching: en vez de responder 'no puedo dar rankings', el matcher agarra cualquier recurso que comparta una palabra generica ('alumno'/'nota') con la pregunta. Misma familia que P4/P6/P14/P29.</t>
   </si>
   <si>
     <t>BUG #2 — El matcher engancha un recurso por palabra generica y se salta el quiz/tarea/analitica.
@@ -738,7 +738,7 @@
     <t>2 cursos: (1) ADGD0208: respuesta analitica correcta - 'no hay datos de calificaciones de Marcos Del Saz... no se han registrado calificaciones', con insights; honesta y usa el nombre. (2) Otro curso: engancho el PDF 'NOTA INFORMATIVA DIRIGIDA A LOS PARTICIPANTES' por el token 'nota'. Metadatos, mal.</t>
   </si>
   <si>
-    <t>Inconsistente por el bug de matching: si hay un recurso con 'nota' en el nombre, lo engancha; si no, va por analitica (curso 1, respuesta decente). El matching por palabra generica ('nota') vuelve a fallar. Ademas consultar la nota de un alumno por nombre roza PRIVACIDAD: decidir si debe permitirse y con que permisos.</t>
+    <t>[Email eliminado en #6.2 (v1.1.9). Consulta de nota individual por nombre ahora gateada por permiso moodle/grade:viewall.]  Inconsistente por el bug de matching: si hay un recurso con 'nota' en el nombre, lo engancha; si no, va por analitica (curso 1, respuesta decente). El matching por palabra generica ('nota') vuelve a fallar. Ademas consultar la nota de un alumno por nombre roza PRIVACIDAD: decidir si debe permitirse y con que permisos.</t>
   </si>
   <si>
     <t>MISMO fix que P30 (matching por 'nota'/'alumno'). Copia y usa el prompt de P30. Adicional (privacidad): decide la politica para consultar la nota de un alumno concreto por nombre; si se permite, usa get_grades_and_quizzes filtrado por usuario respetando capacidades de Moodle; si no, responde que no se consultan notas individuales.</t>
@@ -753,7 +753,7 @@
     <t>BOTON 'En riesgo' en 2 cursos: Curso 1 BIEN (2 en riesgo: Marcos Del Saz, Alumno SEPE, con razon/progreso/accion/insights/recomendaciones). Curso 2 MAL: el MISMO boton engancha el PDF 'Manual de uso de la plataforma para el estudiante' (MANUAL_ESTUDIANTE_SEPE.pdf) por el token 'estudiante'.</t>
   </si>
   <si>
-    <t>CORRECCION: ambas pruebas fueron con el BOTON. El boton NO tiene handler propio: inyecta una pregunta en lenguaje natural que pasa por el mismo pipeline y es vulnerable al matcher. La funcion 'en riesgo' EXISTE y es muy buena, pero solo acierta cuando ningun recurso del curso choca con las palabras de la pregunta ('alumno/estudiante'). En cursos con un PDF tipo 'Manual del estudiante' o 'Guia del alumno', hasta el boton falla. Esto eleva la prioridad del fix del matcher: afecta incluso a las funciones accesibles por boton.</t>
+    <t>[✓✓ RE-VERIFICADA con Claude (v1.2.4): 3 de 12 en riesgo, razon/accion/progreso por alumno, SIN email (privacidad #6.2 OK). Distingue 'intento sin nota' vs 'sin intento'.]  CORRECCION: ambas pruebas fueron con el BOTON. El boton NO tiene handler propio: inyecta una pregunta en lenguaje natural que pasa por el mismo pipeline y es vulnerable al matcher. La funcion 'en riesgo' EXISTE y es muy buena, pero solo acierta cuando ningun recurso del curso choca con las palabras de la pregunta ('alumno/estudiante'). En cursos con un PDF tipo 'Manual del estudiante' o 'Guia del alumno', hasta el boton falla. Esto eleva la prioridad del fix del matcher: afecta incluso a las funciones accesibles por boton.</t>
   </si>
   <si>
     <t>Contexto: Plugin de Moodle `block_pulso`. Ficheros: chat_simple_view.php (botones), classes/rag_retriever.php, classes/chat_pipeline.php.
@@ -773,7 +773,7 @@
     <t>Ambos cursos: 'El documento no contiene/proporciona informacion sobre un ranking de notas de los alumnos.' Modo documento.</t>
   </si>
   <si>
-    <t>Hueco de funcionalidad (no hay ranking) + enrutado a modo documento (por 'nota'/'alumnos'). El dato base (grades_and_quizzes) existe.</t>
+    <t>[✓ RESUELTA + RE-VERIFICADA (#6.2 + Claude v1.2.4): ranking renderiza como tarjetas (Maria Petra 100% rango 1, 6 empatados a 93.33%), SIN emails (privacidad OK). Era la que salia en JSON crudo antes del fix del prefill.]  [APLICADO #6.2 (v1.1.9): ranking pre-calculado + privacidad (solo con moodle/grade:viewall se ven nombres/notas individuales; sin permiso, solo agregados). Email eliminado. PENDIENTE verificar con rol profesor y rol alumno.]  Hueco de funcionalidad (no hay ranking) + enrutado a modo documento (por 'nota'/'alumnos'). El dato base (grades_and_quizzes) existe.</t>
   </si>
   <si>
     <t>Contexto: Plugin de Moodle `block_pulso`. Fichero: classes/rag_retriever.php (+ data_retriever.php si se implementa la funcion).
@@ -861,7 +861,7 @@
     <t>Identifico el recurso 'Cuento' (el-pais-de-la-geometria...docx) pero solo dio metadatos, no el contenido. Seguimiento 'resumen de su contenido' engancho OTRA actividad (MF0233/UF0323 Paso 2 'Resumen', tarea de presentaciones) por la palabra 'resumen'.</t>
   </si>
   <si>
-    <t>Limitacion esperada: content_extractor solo extrae text/*, .ipynb y PDF; Office (.docx/.pptx/.xlsx) NO -&gt; solo metadatos. Ademas, el seguimiento muestra de nuevo el bug de matching ('resumen' engancha una actividad llamada 'Resumen'). Candidato a MEJORA: soporte de extraccion .docx.</t>
+    <t>[APLICADO #6.1 (v1.1.8): extraccion de .docx/.pptx via ZipArchive (word/document.xml y ppt/slides/slideN.xml). PENDIENTE verificar: 'resume el documento Cuento' -&gt; contenido real.]  Limitacion esperada: content_extractor solo extrae text/*, .ipynb y PDF; Office (.docx/.pptx/.xlsx) NO -&gt; solo metadatos. Ademas, el seguimiento muestra de nuevo el bug de matching ('resumen' engancha una actividad llamada 'Resumen'). Candidato a MEJORA: soporte de extraccion .docx.</t>
   </si>
   <si>
     <t>Contexto: Plugin de Moodle `block_pulso`. Fichero: classes/content_extractor.php, funcion `extract_resource()`.
@@ -1070,7 +1070,7 @@
     <t>Respondio a nivel de CURSO (ADGD0208, 4 secciones), no del SCORM. Describio cada seccion infiriendo por el titulo con lenguaje de suposicion ('probablemente cubre', 'posiblemente con un enfoque'). No accedio al contenido del SCORM.</t>
   </si>
   <si>
-    <t>OJO: Phia y Pulso AI se probaron en CURSOS DISTINTOS (Phia en un SCORM de 'cooperativas de trabajo'; Pulso en ADGD0208 RRHH). Es una comparacion de CAPACIDAD, no de misma respuesta. Conclusion valida igualmente: Phia accede al contenido del SCORM y da objetivos de aprendizaje reales; Pulso trabaja a nivel de curso e infiere el contenido por los nombres de seccion ('probablemente/posiblemente') -&gt; riesgo de alucinacion. Para una comparacion 1:1 habria que apuntar ambos al mismo SCORM.</t>
+    <t>[APLICADO #6.3 (v1.1.10): indexacion de contenido SCORM (lee HTML descomprimido por Moodle, orden via imsmanifest). PENDIENTE: reindexar curso y verificar 'de que trata esta unidad' sobre un SCORM HTML. Limitacion: SCORM Articulate/Storyline (JS) dara aviso claro.]  OJO: Phia y Pulso AI se probaron en CURSOS DISTINTOS (Phia en un SCORM de 'cooperativas de trabajo'; Pulso en ADGD0208 RRHH). Es una comparacion de CAPACIDAD, no de misma respuesta. Conclusion valida igualmente: Phia accede al contenido del SCORM y da objetivos de aprendizaje reales; Pulso trabaja a nivel de curso e infiere el contenido por los nombres de seccion ('probablemente/posiblemente') -&gt; riesgo de alucinacion. Para una comparacion 1:1 habria que apuntar ambos al mismo SCORM.</t>
   </si>
   <si>
     <t>Contexto: Plugin de Moodle `block_pulso`. Comparativa con otro plugin (Phia) que SI lee el contenido de los SCORM. Ficheros: classes/content_extractor.php, classes/system_prompt_designer.php, classes/rag_retriever.php.
@@ -1096,7 +1096,7 @@
     <t>'Investigacion cuantitativa': explicacion correcta pero GENERICA (metodos, datos numericos, estadistica...), sacada del conocimiento general del modelo, no del contenido del SCORM/curso.</t>
   </si>
   <si>
-    <t>No falla (da explicacion valida) pero NO esta anclada en el material del curso. Para conceptos generales cuela; para conceptos con enfoque propio del curso o especificos, seria generico o podria no coincidir con lo que ensena el temario. No puede citar el material. [SEGUIMIENTO ROTO: al preguntar despues '¿cuales son los metodos mas comunes en investigacion cuantitativa?', engancho el PDF 'Principios eticos en la investigacion cientifica' por compartir 'investigacion/cientifica'. Aunque la explicacion inicial es decente, el seguimiento se rompe por el matcher (bug #2). Impide conversacion fluida sobre un tema -&gt; refuerza la prioridad del fix de P30.]</t>
+    <t>[APLICADO #6.3 (v1.1.10): mismo fix de indexacion SCORM. PENDIENTE verificar 'explicame un concepto' sobre un SCORM HTML tras reindexar.]  No falla (da explicacion valida) pero NO esta anclada en el material del curso. Para conceptos generales cuela; para conceptos con enfoque propio del curso o especificos, seria generico o podria no coincidir con lo que ensena el temario. No puede citar el material. [SEGUIMIENTO ROTO: al preguntar despues '¿cuales son los metodos mas comunes en investigacion cuantitativa?', engancho el PDF 'Principios eticos en la investigacion cientifica' por compartir 'investigacion/cientifica'. Aunque la explicacion inicial es decente, el seguimiento se rompe por el matcher (bug #2). Impide conversacion fluida sobre un tema -&gt; refuerza la prioridad del fix de P30.]</t>
   </si>
   <si>
     <t>Ver P55: indexar el contenido del SCORM (content_extractor.php). Con eso, las explicaciones de conceptos pasarian de 'genericas del modelo' a 'ancladas en el material del curso', y podria citar/ajustarse al temario.</t>
@@ -1410,16 +1410,22 @@
     <xf numFmtId="0" fontId="17" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1428,13 +1434,7 @@
     <xf numFmtId="0" fontId="20" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1763,7 +1763,7 @@
       </c>
     </row>
     <row r="5" spans="2:6" ht="24" customHeight="1">
-      <c r="B5" s="32" t="s">
+      <c r="B5" s="31" t="s">
         <v>2</v>
       </c>
       <c r="C5" s="41"/>
@@ -1800,7 +1800,7 @@
       </c>
     </row>
     <row r="9" spans="2:6">
-      <c r="B9" s="38" t="s">
+      <c r="B9" s="33" t="s">
         <v>11</v>
       </c>
       <c r="C9" s="41"/>
@@ -1809,7 +1809,7 @@
       <c r="F9" s="41"/>
     </row>
     <row r="11" spans="2:6" ht="24" customHeight="1">
-      <c r="B11" s="32" t="s">
+      <c r="B11" s="31" t="s">
         <v>12</v>
       </c>
       <c r="C11" s="41"/>
@@ -1818,7 +1818,7 @@
       <c r="F11" s="41"/>
     </row>
     <row r="12" spans="2:6" ht="15.95" customHeight="1">
-      <c r="B12" s="35" t="s">
+      <c r="B12" s="37" t="s">
         <v>13</v>
       </c>
       <c r="C12" s="42"/>
@@ -1827,7 +1827,7 @@
       <c r="F12" s="43"/>
     </row>
     <row r="13" spans="2:6" ht="45.95" customHeight="1">
-      <c r="B13" s="37" t="s">
+      <c r="B13" s="36" t="s">
         <v>14</v>
       </c>
       <c r="C13" s="42"/>
@@ -1836,7 +1836,7 @@
       <c r="F13" s="43"/>
     </row>
     <row r="14" spans="2:6" ht="15.95" customHeight="1">
-      <c r="B14" s="35" t="s">
+      <c r="B14" s="37" t="s">
         <v>15</v>
       </c>
       <c r="C14" s="42"/>
@@ -1845,7 +1845,7 @@
       <c r="F14" s="43"/>
     </row>
     <row r="15" spans="2:6" ht="45.95" customHeight="1">
-      <c r="B15" s="37" t="s">
+      <c r="B15" s="36" t="s">
         <v>16</v>
       </c>
       <c r="C15" s="42"/>
@@ -1854,7 +1854,7 @@
       <c r="F15" s="43"/>
     </row>
     <row r="16" spans="2:6" ht="15.95" customHeight="1">
-      <c r="B16" s="31" t="s">
+      <c r="B16" s="35" t="s">
         <v>17</v>
       </c>
       <c r="C16" s="42"/>
@@ -1872,7 +1872,7 @@
       <c r="F17" s="43"/>
     </row>
     <row r="18" spans="2:6" ht="15.95" customHeight="1">
-      <c r="B18" s="31" t="s">
+      <c r="B18" s="35" t="s">
         <v>19</v>
       </c>
       <c r="C18" s="42"/>
@@ -1890,7 +1890,7 @@
       <c r="F19" s="43"/>
     </row>
     <row r="20" spans="2:6" ht="15.95" customHeight="1">
-      <c r="B20" s="31" t="s">
+      <c r="B20" s="35" t="s">
         <v>21</v>
       </c>
       <c r="C20" s="42"/>
@@ -1908,7 +1908,7 @@
       <c r="F21" s="43"/>
     </row>
     <row r="22" spans="2:6" ht="15.95" customHeight="1">
-      <c r="B22" s="33" t="s">
+      <c r="B22" s="39" t="s">
         <v>23</v>
       </c>
       <c r="C22" s="42"/>
@@ -1917,7 +1917,7 @@
       <c r="F22" s="43"/>
     </row>
     <row r="23" spans="2:6" ht="45.95" customHeight="1">
-      <c r="B23" s="36" t="s">
+      <c r="B23" s="38" t="s">
         <v>24</v>
       </c>
       <c r="C23" s="42"/>
@@ -1926,7 +1926,7 @@
       <c r="F23" s="43"/>
     </row>
     <row r="25" spans="2:6" ht="24" customHeight="1">
-      <c r="B25" s="32" t="s">
+      <c r="B25" s="31" t="s">
         <v>25</v>
       </c>
       <c r="C25" s="41"/>
@@ -1935,7 +1935,7 @@
       <c r="F25" s="41"/>
     </row>
     <row r="26" spans="2:6" ht="45.95" customHeight="1">
-      <c r="B26" s="39" t="s">
+      <c r="B26" s="32" t="s">
         <v>26</v>
       </c>
       <c r="C26" s="41"/>
@@ -1944,7 +1944,7 @@
       <c r="F26" s="41"/>
     </row>
     <row r="28" spans="2:6" ht="24" customHeight="1">
-      <c r="B28" s="32" t="s">
+      <c r="B28" s="31" t="s">
         <v>27</v>
       </c>
       <c r="C28" s="41"/>
@@ -1953,7 +1953,7 @@
       <c r="F28" s="41"/>
     </row>
     <row r="29" spans="2:6" ht="45.95" customHeight="1">
-      <c r="B29" s="38" t="s">
+      <c r="B29" s="33" t="s">
         <v>28</v>
       </c>
       <c r="C29" s="41"/>
@@ -1963,6 +1963,9 @@
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="B22:F22"/>
+    <mergeCell ref="B18:F18"/>
+    <mergeCell ref="B21:F21"/>
     <mergeCell ref="B5:F5"/>
     <mergeCell ref="B26:F26"/>
     <mergeCell ref="B29:F29"/>
@@ -1979,9 +1982,6 @@
     <mergeCell ref="B13:F13"/>
     <mergeCell ref="B16:F16"/>
     <mergeCell ref="B25:F25"/>
-    <mergeCell ref="B22:F22"/>
-    <mergeCell ref="B18:F18"/>
-    <mergeCell ref="B21:F21"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3214,8 +3214,8 @@
       <c r="D42" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="E42" s="12" t="s">
-        <v>9</v>
+      <c r="E42" s="11" t="s">
+        <v>7</v>
       </c>
       <c r="F42" s="15" t="s">
         <v>226</v>

</xml_diff>

<commit_message>
Cierra el QA: reprueba los fallos tras v1.14.1
</commit_message>
<xml_diff>
--- a/Pulso_AI_matriz_evaluacion.xlsx
+++ b/Pulso_AI_matriz_evaluacion.xlsx
@@ -1495,9 +1495,9 @@
           <t>Bien</t>
         </is>
       </c>
-      <c r="E6" s="16" t="inlineStr">
-        <is>
-          <t>Mal</t>
+      <c r="E6" s="13" t="inlineStr">
+        <is>
+          <t>Bien</t>
         </is>
       </c>
       <c r="F6" s="19" t="inlineStr">
@@ -1507,7 +1507,7 @@
       </c>
       <c r="G6" s="14" t="inlineStr">
         <is>
-          <t>[RONDA 3 — curso SANS0001 (id 92), v1.11.0, Claude Sonnet 5] 'Que actividades hay en la seccion RECURSOS' devolvio UN solo recurso (MATERIAL 1) en vez de listar los ~12 de la seccion. BUG VIVO.  ||  BUG de enrutado: al pedir 'qué actividades hay en la sección X', la detección de label (resolve_direct_label_in_section_query) intercepta antes que el listado de la sección. La intención 'listar actividades de sección' debería tener prioridad sobre el match de label. A revisar en rag_retriever.php.</t>
+          <t>[RONDA 5: control repasado, SIGUE BIEN] [RONDA 4 - 07/09/2026, curso SANS0001 (id 92), tras los arreglos] ARREGLADO. Lista las 11 actividades de la seccion RECURSOS con su tipo (10 RESOURCE + 1 PAGE). Antes devolvia solo MATERIAL 1.  ||  [RONDA 3 — curso SANS0001 (id 92), v1.11.0, Claude Sonnet 5] 'Que actividades hay en la seccion RECURSOS' devolvio UN solo recurso (MATERIAL 1) en vez de listar los ~12 de la seccion. BUG VIVO.  ||  BUG de enrutado: al pedir 'qué actividades hay en la sección X', la detección de label (resolve_direct_label_in_section_query) intercepta antes que el listado de la sección. La intención 'listar actividades de sección' debería tener prioridad sobre el match de label. A revisar en rag_retriever.php.</t>
         </is>
       </c>
       <c r="H6" s="21" t="inlineStr">
@@ -1542,9 +1542,9 @@
           <t>Bien</t>
         </is>
       </c>
-      <c r="E7" s="16" t="inlineStr">
-        <is>
-          <t>Mal</t>
+      <c r="E7" s="13" t="inlineStr">
+        <is>
+          <t>Bien</t>
         </is>
       </c>
       <c r="F7" s="19" t="inlineStr">
@@ -1554,7 +1554,7 @@
       </c>
       <c r="G7" s="14" t="inlineStr">
         <is>
-          <t>[RONDA 3 — curso SANS0001 (id 92), v1.11.0, Claude Sonnet 5] 'Que hay en el tema 2' lo interpreto como el RECURSO 'MIC Tema 2' (colision de nombre) en vez de la Seccion 2. BUG del matcher.  ||  Correcto por número de tema. Contrasta con P4: por número lista bien la sección; por nombre se desvió a la etiqueta. Confirma que el bug de P4 está en el match por nombre de sección.</t>
+          <t>[RONDA 5: control repasado, SIGUE BIEN] [RONDA 4 - 07/09/2026, curso SANS0001 (id 92), tras los arreglos] ARREGLADO. 'Que hay en el tema 2' -&gt; Seccion 2 'Diplomas' (1 actividad, CUSTOMCERT APROVECHAMIENTO). Ya no engancha el recurso homonimo 'MIC Tema 2'.  ||  [RONDA 3 — curso SANS0001 (id 92), v1.11.0, Claude Sonnet 5] 'Que hay en el tema 2' lo interpreto como el RECURSO 'MIC Tema 2' (colision de nombre) en vez de la Seccion 2. BUG del matcher.  ||  Correcto por número de tema. Contrasta con P4: por número lista bien la sección; por nombre se desvió a la etiqueta. Confirma que el bug de P4 está en el match por nombre de sección.</t>
         </is>
       </c>
       <c r="H7" s="21" t="n"/>
@@ -1786,7 +1786,7 @@
       </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
-          <t>[RONDA 3 — curso SANS0001 (id 92), v1.11.0, Claude Sonnet 5] 15 preguntas + boton de enlace.  ||  [✓ RECUPERADA con fix #2 (v1.1.4): 'tiene 15 preguntas'. El match exacto del quiz gana; ya no lo secuestra un PDF.]  Correcto, ruta directa. El curso sí tiene un quiz real ('Cuestionario tipo test'). [OJO: tras el fix #1, en cursos con un recurso cuyo nombre contiene 'tipo'/'test'/'cuestionario', esta pregunta la intercepta el bug #2 (el matcher agarra el recurso antes que el quiz) y falla con 'no aparece en el documento'. NO es regresion del fix #1 (commit solo toco la regex + version; la logica de conteo esta intacta). Se recupera con el fix #2.]</t>
+          <t>[RONDA 5: control repasado, SIGUE BIEN] [RONDA 3 — curso SANS0001 (id 92), v1.11.0, Claude Sonnet 5] 15 preguntas + boton de enlace.  ||  [✓ RECUPERADA con fix #2 (v1.1.4): 'tiene 15 preguntas'. El match exacto del quiz gana; ya no lo secuestra un PDF.]  Correcto, ruta directa. El curso sí tiene un quiz real ('Cuestionario tipo test'). [OJO: tras el fix #1, en cursos con un recurso cuyo nombre contiene 'tipo'/'test'/'cuestionario', esta pregunta la intercepta el bug #2 (el matcher agarra el recurso antes que el quiz) y falla con 'no aparece en el documento'. NO es regresion del fix #1 (commit solo toco la regex + version; la logica de conteo esta intacta). Se recupera con el fix #2.]</t>
         </is>
       </c>
       <c r="H14" s="21" t="n"/>
@@ -2120,9 +2120,9 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E23" s="15" t="inlineStr">
-        <is>
-          <t>Regular</t>
+      <c r="E23" s="13" t="inlineStr">
+        <is>
+          <t>Bien</t>
         </is>
       </c>
       <c r="F23" s="19" t="inlineStr">
@@ -2132,7 +2132,7 @@
       </c>
       <c r="G23" s="14" t="inlineStr">
         <is>
-          <t>[RONDA 3 — curso SANS0001 (id 92), v1.11.0, Claude Sonnet 5] 'Resumeme el curso' devolvio un resumen ANALITICO (4 secciones, 13 alumnos, tasa aprobacion) en vez del contenido/temario. Se desvia.  ||  Correcto, ruta RAG. Consistente con P17. Buen tono de resumen.</t>
+          <t>[RONDA 4 - 07/09/2026, curso SANS0001 (id 92), tras los arreglos] ARREGLADO. Resumen por estructura + cierra con el TEMARIO real (definicion y enfoque, objetividad, cuantitativo vs cualitativo, etica, elaboracion de proyectos). Ya no mete analitica.  ||  [RONDA 3 — curso SANS0001 (id 92), v1.11.0, Claude Sonnet 5] 'Resumeme el curso' devolvio un resumen ANALITICO (4 secciones, 13 alumnos, tasa aprobacion) en vez del contenido/temario. Se desvia.  ||  Correcto, ruta RAG. Consistente con P17. Buen tono de resumen.</t>
         </is>
       </c>
       <c r="H23" s="21" t="n"/>
@@ -2212,7 +2212,7 @@
       </c>
       <c r="G25" s="14" t="inlineStr">
         <is>
-          <t>[RONDA 3 — curso SANS0001 (id 92), v1.11.0, Claude Sonnet 5] Con contexto limpio resumio el contenido REAL del PDF (poblacion, muestra, variables) + boton. OJO: con contexto sucio fallaba.  ||  Validado indirectamente vía P49. La extraccion y el resumen de PDFs funcionan.</t>
+          <t>[RONDA 5: control repasado, SIGUE BIEN] [RONDA 3 — curso SANS0001 (id 92), v1.11.0, Claude Sonnet 5] Con contexto limpio resumio el contenido REAL del PDF (poblacion, muestra, variables) + boton. OJO: con contexto sucio fallaba.  ||  Validado indirectamente vía P49. La extraccion y el resumen de PDFs funcionan.</t>
         </is>
       </c>
       <c r="H25" s="21" t="n"/>
@@ -2238,9 +2238,9 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E26" s="15" t="inlineStr">
-        <is>
-          <t>Regular</t>
+      <c r="E26" s="13" t="inlineStr">
+        <is>
+          <t>Bien</t>
         </is>
       </c>
       <c r="F26" s="19" t="inlineStr">
@@ -2250,7 +2250,7 @@
       </c>
       <c r="G26" s="14" t="inlineStr">
         <is>
-          <t>[RONDA 3 — curso SANS0001 (id 92), v1.11.0, Claude Sonnet 5] 'Que dice el documento X sobre Y' devolvio solo METADATOS + enlace, sin responder. Bug de fraseo NUNCA arreglado (mismo que P7 antiguo).  ||  Mismo bug de fraseo que P7. 'Que dice el documento X sobre Y' no dispara la extraccion de contenido para recursos, cae a metadatos. Incoherente: P49 ('resumen de ese pdf') SI extrajo contenido pero esta no. El triggering de content_mode depende demasiado del fraseo exacto.</t>
+          <t>[RONDA 4 - 07/09/2026, curso SANS0001 (id 92), tras los arreglos] ARREGLADO. Devuelve el CONTENIDO del PDF (definicion, objetividad, cuantificacion, poblacion/muestra/variables) en vez de metadatos. Acerto con 4 mensajes previos en contexto.  ||  [RONDA 3 — curso SANS0001 (id 92), v1.11.0, Claude Sonnet 5] 'Que dice el documento X sobre Y' devolvio solo METADATOS + enlace, sin responder. Bug de fraseo NUNCA arreglado (mismo que P7 antiguo).  ||  Mismo bug de fraseo que P7. 'Que dice el documento X sobre Y' no dispara la extraccion de contenido para recursos, cae a metadatos. Incoherente: P49 ('resumen de ese pdf') SI extrajo contenido pero esta no. El triggering de content_mode depende demasiado del fraseo exacto.</t>
         </is>
       </c>
       <c r="H26" s="21" t="inlineStr">
@@ -2771,9 +2771,9 @@
           <t>Mal</t>
         </is>
       </c>
-      <c r="E40" s="50" t="inlineStr">
-        <is>
-          <t>Mal</t>
+      <c r="E40" s="13" t="inlineStr">
+        <is>
+          <t>Bien</t>
         </is>
       </c>
       <c r="F40" s="19" t="inlineStr">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="G40" s="14" t="inlineStr">
         <is>
-          <t>[SIN RE-TEST EN RONDA 3 - el veredicto de la columna Resultado es el de la evaluacion original y puede estar obsoleto] [Email eliminado en #6.2 (v1.1.9). Consulta de nota individual por nombre ahora gateada por permiso moodle/grade:viewall.]  Inconsistente por el bug de matching: si hay un recurso con 'nota' en el nombre, lo engancha; si no, va por analitica (curso 1, respuesta decente). El matching por palabra generica ('nota') vuelve a fallar. Ademas consultar la nota de un alumno por nombre roza PRIVACIDAD: decidir si debe permitirse y con que permisos.</t>
+          <t>[RONDA 4 - 07/09/2026, curso SANS0001 (id 92), tras los arreglos] MARIA PETRA GORDILLO GONZALEZ 10/10 (100%), con nota de corte, resultado, insights y recomendaciones. Sin email.  ||  [Email eliminado en #6.2 (v1.1.9). Consulta de nota individual por nombre ahora gateada por permiso moodle/grade:viewall.]  Inconsistente por el bug de matching: si hay un recurso con 'nota' en el nombre, lo engancha; si no, va por analitica (curso 1, respuesta decente). El matching por palabra generica ('nota') vuelve a fallar. Ademas consultar la nota de un alumno por nombre roza PRIVACIDAD: decidir si debe permitirse y con que permisos.</t>
         </is>
       </c>
       <c r="H40" s="21" t="inlineStr">
@@ -2923,9 +2923,9 @@
           <t>Mal</t>
         </is>
       </c>
-      <c r="E44" s="50" t="inlineStr">
-        <is>
-          <t>Regular</t>
+      <c r="E44" s="13" t="inlineStr">
+        <is>
+          <t>Bien</t>
         </is>
       </c>
       <c r="F44" s="19" t="inlineStr">
@@ -2935,7 +2935,7 @@
       </c>
       <c r="G44" s="14" t="inlineStr">
         <is>
-          <t>[SIN RE-TEST EN RONDA 3 - el veredicto de la columna Resultado es el de la evaluacion original y puede estar obsoleto] Regular. Limitacion de ventana temporal confirmada: el plugin solo lee 7 dias de logs (get_unified_course_context ..., 7), pero el curso 1 presenta esos datos como 'lo que va del mes' (hoy 10-jul) -&gt; ENGANOSO, faltan dias 1-3. El motor de analitica de accesos funciona; el problema es el alcance temporal y el etiquetado. Curso 2 responde con no-dato amable (inconsistencia entre cursos).</t>
+          <t>[RONDA 4 - 07/09/2026, curso SANS0001 (id 92), tras los arreglos] 81 accesos en septiembre, rango 2-7/09. Honesto sobre la ventana de 7 dias de logs y distingue admin (Leonardo 56, Marcos 24) de alumnos (0).  ||  Regular. Limitacion de ventana temporal confirmada: el plugin solo lee 7 dias de logs (get_unified_course_context ..., 7), pero el curso 1 presenta esos datos como 'lo que va del mes' (hoy 10-jul) -&gt; ENGANOSO, faltan dias 1-3. El motor de analitica de accesos funciona; el problema es el alcance temporal y el etiquetado. Curso 2 responde con no-dato amable (inconsistencia entre cursos).</t>
         </is>
       </c>
       <c r="H44" s="21" t="inlineStr">
@@ -3008,9 +3008,9 @@
           <t>Mal</t>
         </is>
       </c>
-      <c r="E46" s="51" t="inlineStr">
-        <is>
-          <t>Regular</t>
+      <c r="E46" s="13" t="inlineStr">
+        <is>
+          <t>Bien</t>
         </is>
       </c>
       <c r="F46" s="19" t="inlineStr">
@@ -3020,7 +3020,7 @@
       </c>
       <c r="G46" s="14" t="inlineStr">
         <is>
-          <t>[SIN RE-TEST EN RONDA 3 - el veredicto de la columna Resultado es el de la evaluacion original y puede estar obsoleto] [✓ ENRUTADO ARREGLADO (v1.1.5/1.1.6): ya no engancha un PDF, da los accesos reales. Queda la ventana temporal de ~7 dias para 'ultimas semanas' -&gt; mejora P35.]  [PARCIAL con fix #3 (v1.1.5): resuelta la contaminacion de historial. Queda la ventana temporal de 7 dias para 'ultimas semanas' (ver fix P35). Re-test recomendado.]  Mal por dos posibles causas: (1) la palabra 'actividad' dispara la resolucion de una actividad; (2) contaminacion del history-hint (Guia del alumno salio en P30/P31/P33 de este chat). Ademas, aunque llegara a analitica, la ventana de 7 dias se quedaria corta para 'ultimas semanas'. Sugerido: repetir en chat NUEVO para descartar history-hint.</t>
+          <t>[RONDA 4 - 07/09/2026, curso SANS0001 (id 92), tras los arreglos] 81 accesos entre 2/09 y 7/09, avisando de que el 100% es personal administrativo/tutores y no hay actividad de alumnos.  ||  [✓ ENRUTADO ARREGLADO (v1.1.5/1.1.6): ya no engancha un PDF, da los accesos reales. Queda la ventana temporal de ~7 dias para 'ultimas semanas' -&gt; mejora P35.]  [PARCIAL con fix #3 (v1.1.5): resuelta la contaminacion de historial. Queda la ventana temporal de 7 dias para 'ultimas semanas' (ver fix P35). Re-test recomendado.]  Mal por dos posibles causas: (1) la palabra 'actividad' dispara la resolucion de una actividad; (2) contaminacion del history-hint (Guia del alumno salio en P30/P31/P33 de este chat). Ademas, aunque llegara a analitica, la ventana de 7 dias se quedaria corta para 'ultimas semanas'. Sugerido: repetir en chat NUEVO para descartar history-hint.</t>
         </is>
       </c>
       <c r="H46" s="21" t="inlineStr">
@@ -3066,9 +3066,9 @@
           <t>Mal</t>
         </is>
       </c>
-      <c r="E48" s="50" t="inlineStr">
-        <is>
-          <t>Mal</t>
+      <c r="E48" s="15" t="inlineStr">
+        <is>
+          <t>Regular</t>
         </is>
       </c>
       <c r="F48" s="19" t="inlineStr">
@@ -3078,7 +3078,7 @@
       </c>
       <c r="G48" s="14" t="inlineStr">
         <is>
-          <t>[SIN RE-TEST EN RONDA 3 - el veredicto de la columna Resultado es el de la evaluacion original y puede estar obsoleto] [PARCIAL con fix #3 (v1.1.5): al nombrar el foro ya NO arrastra 'Guia del alumno'; deberia resolver el foro. PERO el contenido de foros sigue sin indexarse (mejora #6). Re-test recomendado.]  EVIDENCIA FUERTE de history-hint contaminado: 'Guia del alumno' aparece en P30/P31/P33/P37/P38 del mismo chat. El history-hint queda pegado a un recurso previo y lo devuelve aunque no tenga relacion. Ademas, el contenido de foros NO se indexa en RAG. RECOMENDACION: repetir en chat NUEVO. Bug de history-hint = alta prioridad (relacionado con P14).</t>
+          <t>[RONDA 5 - 07/09/2026, tras v1.14.0 y v1.14.1] SIGUE IGUAL. En frio responde bien (0 discusiones, 0 mensajes + boton). Preguntada tras una respuesta de analitica devuelve OTRA VEZ la tabla de accesos (91 accesos). La contaminacion tras analitica NO se ha arreglado con v1.14.0.  ||  [RONDA 4 - 07/09/2026, curso SANS0001 (id 92), tras los arreglos] Con contexto LIMPIO responde bien (0 discusiones, 0 mensajes, descripcion + boton 'Ir a foro'). Pero preguntado despues de dos respuestas de analitica devolvio la tabla de ACCESOS. Contaminacion residual.  ||  [PARCIAL con fix #3 (v1.1.5): al nombrar el foro ya NO arrastra 'Guia del alumno'; deberia resolver el foro. PERO el contenido de foros sigue sin indexarse (mejora #6). Re-test recomendado.]  EVIDENCIA FUERTE de history-hint contaminado: 'Guia del alumno' aparece en P30/P31/P33/P37/P38 del mismo chat. El history-hint queda pegado a un recurso previo y lo devuelve aunque no tenga relacion. Ademas, el contenido de foros NO se indexa en RAG. RECOMENDACION: repetir en chat NUEVO. Bug de history-hint = alta prioridad (relacionado con P14).</t>
         </is>
       </c>
       <c r="H48" s="21" t="inlineStr">
@@ -3108,9 +3108,9 @@
           <t>Mal</t>
         </is>
       </c>
-      <c r="E49" s="50" t="inlineStr">
-        <is>
-          <t>Mal</t>
+      <c r="E49" s="49" t="inlineStr">
+        <is>
+          <t>No aplica</t>
         </is>
       </c>
       <c r="F49" s="19" t="inlineStr">
@@ -3120,7 +3120,7 @@
       </c>
       <c r="G49" s="14" t="inlineStr">
         <is>
-          <t>[SIN RE-TEST EN RONDA 3 - el veredicto de la columna Resultado es el de la evaluacion original y puede estar obsoleto] [APLICADO #6.1 (v1.1.8): extraccion de .docx/.pptx via ZipArchive (word/document.xml y ppt/slides/slideN.xml). PENDIENTE verificar: 'resume el documento Cuento' -&gt; contenido real.]  Limitacion esperada: content_extractor solo extrae text/*, .ipynb y PDF; Office (.docx/.pptx/.xlsx) NO -&gt; solo metadatos. Ademas, el seguimiento muestra de nuevo el bug de matching ('resumen' engancha una actividad llamada 'Resumen'). Candidato a MEJORA: soporte de extraccion .docx.</t>
+          <t>[RONDA 4 - 07/09/2026, curso SANS0001 (id 92), tras los arreglos] El curso no tiene ningun .docx: los 10 recursos son PDF y 1 es una pagina Moodle. Verificado en el DOM del curso.  ||  [APLICADO #6.1 (v1.1.8): extraccion de .docx/.pptx via ZipArchive (word/document.xml y ppt/slides/slideN.xml). PENDIENTE verificar: 'resume el documento Cuento' -&gt; contenido real.]  Limitacion esperada: content_extractor solo extrae text/*, .ipynb y PDF; Office (.docx/.pptx/.xlsx) NO -&gt; solo metadatos. Ademas, el seguimiento muestra de nuevo el bug de matching ('resumen' engancha una actividad llamada 'Resumen'). Candidato a MEJORA: soporte de extraccion .docx.</t>
         </is>
       </c>
       <c r="H49" s="21" t="inlineStr">
@@ -3155,7 +3155,7 @@
           <t>Mal</t>
         </is>
       </c>
-      <c r="E50" s="50" t="inlineStr">
+      <c r="E50" s="49" t="inlineStr">
         <is>
           <t>No aplica</t>
         </is>
@@ -3163,7 +3163,7 @@
       <c r="F50" s="19" t="n"/>
       <c r="G50" s="14" t="inlineStr">
         <is>
-          <t>[SIN RE-TEST EN RONDA 3 - el veredicto de la columna Resultado es el de la evaluacion original y puede estar obsoleto] No hay .pptx en el curso. Nota: aunque lo hubiera, seria Mal (Office no se extrae, igual que P39 .docx). Mejora opcional: soporte extraccion .pptx.</t>
+          <t>[RONDA 4 - 07/09/2026, curso SANS0001 (id 92), tras los arreglos] El curso no tiene ningun .pptx. Verificado en el DOM del curso.  ||  No hay .pptx en el curso. Nota: aunque lo hubiera, seria Mal (Office no se extrae, igual que P39 .docx). Mejora opcional: soporte extraccion .pptx.</t>
         </is>
       </c>
       <c r="H50" s="21" t="n"/>
@@ -3189,7 +3189,7 @@
           <t>Mal</t>
         </is>
       </c>
-      <c r="E51" s="50" t="inlineStr">
+      <c r="E51" s="49" t="inlineStr">
         <is>
           <t>No aplica</t>
         </is>
@@ -3197,7 +3197,7 @@
       <c r="F51" s="19" t="n"/>
       <c r="G51" s="14" t="inlineStr">
         <is>
-          <t>[SIN RE-TEST EN RONDA 3 - el veredicto de la columna Resultado es el de la evaluacion original y puede estar obsoleto] No hay PDF escaneado en el curso. Comportamiento esperado si lo hubiera: Mal, haria falta OCR (no soportado). Distinto del PDF de mates (ese SI tenia texto, ver P22).</t>
+          <t>[RONDA 4 - 07/09/2026, curso SANS0001 (id 92), tras los arreglos] No se ha identificado ningun PDF escaneado en el curso; la extraccion funciona bien en los PDF de texto (P20, P22, P23, P49).  ||  No hay PDF escaneado en el curso. Comportamiento esperado si lo hubiera: Mal, haria falta OCR (no soportado). Distinto del PDF de mates (ese SI tenia texto, ver P22).</t>
         </is>
       </c>
       <c r="H51" s="21" t="n"/>
@@ -3277,7 +3277,7 @@
           <t>Mal</t>
         </is>
       </c>
-      <c r="E54" s="50" t="inlineStr">
+      <c r="E54" s="13" t="inlineStr">
         <is>
           <t>Bien</t>
         </is>
@@ -3289,7 +3289,7 @@
       </c>
       <c r="G54" s="14" t="inlineStr">
         <is>
-          <t>[SIN RE-TEST EN RONDA 3 - el veredicto de la columna Resultado es el de la evaluacion original y puede estar obsoleto] Bien y MUY revelador: el ingles funciona porque las keywords problematicas de la linea 1622 estan en espanol ('nota media'); 'how many passed' no matchea esa regex y va limpio a analitica. Confirma que el bug de P12/P25 es la regex en espanol. NOTA PRIVACIDAD: expone nombres+notas individuales (ver P32).</t>
+          <t>[RONDA 4 - 07/09/2026, curso SANS0001 (id 92), tras los arreglos] Responde en INGLES: '9 of 13 students have passed the quiz (69%)', desglosando 2 sin calificar y 2 sin intentar.  ||  Bien y MUY revelador: el ingles funciona porque las keywords problematicas de la linea 1622 estan en espanol ('nota media'); 'how many passed' no matchea esa regex y va limpio a analitica. Confirma que el bug de P12/P25 es la regex en espanol. NOTA PRIVACIDAD: expone nombres+notas individuales (ver P32).</t>
         </is>
       </c>
       <c r="H54" s="21" t="n"/>
@@ -3315,9 +3315,9 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E55" s="50" t="inlineStr">
-        <is>
-          <t>Bien</t>
+      <c r="E55" s="15" t="inlineStr">
+        <is>
+          <t>Regular</t>
         </is>
       </c>
       <c r="F55" s="19" t="inlineStr">
@@ -3327,7 +3327,7 @@
       </c>
       <c r="G55" s="14" t="inlineStr">
         <is>
-          <t>[SIN RE-TEST EN RONDA 3 - el veredicto de la columna Resultado es el de la evaluacion original y puede estar obsoleto] Mejor de lo esperado: el fraseo alternativo 'en cuantos temas se divide' funciono (probablemente via LLM+contexto de estructura). Se esperaba Regular por depender del literal 'cuantas secciones'.</t>
+          <t>[RONDA 5 - 07/09/2026, tras v1.14.0 y v1.14.1] SIGUE IGUAL. En frio responde bien (4 secciones desglosadas). Tras 'How many students passed?' devuelve la respuesta de aprobados entera. Misma raiz que P38.  ||  [RONDA 4 - 07/09/2026, curso SANS0001 (id 92), tras los arreglos] Con contexto LIMPIO: 4 secciones (formato topics), 3 visibles para alumnos, con desglose de cada una. OJO: preguntado justo despues de una respuesta de analitica devolvio la respuesta anterior (contaminacion).  ||  Mejor de lo esperado: el fraseo alternativo 'en cuantos temas se divide' funciono (probablemente via LLM+contexto de estructura). Se esperaba Regular por depender del literal 'cuantas secciones'.</t>
         </is>
       </c>
       <c r="H55" s="21" t="n"/>
@@ -3353,7 +3353,7 @@
           <t>Mal</t>
         </is>
       </c>
-      <c r="E56" s="52" t="inlineStr">
+      <c r="E56" s="13" t="inlineStr">
         <is>
           <t>Bien</t>
         </is>
@@ -3365,7 +3365,7 @@
       </c>
       <c r="G56" s="14" t="inlineStr">
         <is>
-          <t>[SIN RE-TEST EN RONDA 3 - el veredicto de la columna Resultado es el de la evaluacion original y puede estar obsoleto] [✓ CONFIRMADA (v1.1.6): '9.1 sobre 10' + tabla. Analitica.]  [PROBABLEMENTE RECUPERADA tras fix #1+#2 (v1.1.4), misma raiz que P25/P30 — PENDIENTE de confirmar en chat.]  Fraseo coloquial de nota media. Combina los dos bugs habituales: (1) 'nota...media' captura la intencion de contenido (linea 1622); (2) el matcher engancha 'NOTA INFORMATIVA' por la palabra 'nota'. Distinto de P28 (que dio texto): aqui saco un recurso.</t>
+          <t>[RONDA 4 - 07/09/2026, curso SANS0001 (id 92), tras los arreglos] Nota promedio 9.19/10 (91%) de los alumnos con calificacion registrada.  ||  [✓ CONFIRMADA (v1.1.6): '9.1 sobre 10' + tabla. Analitica.]  [PROBABLEMENTE RECUPERADA tras fix #1+#2 (v1.1.4), misma raiz que P25/P30 — PENDIENTE de confirmar en chat.]  Fraseo coloquial de nota media. Combina los dos bugs habituales: (1) 'nota...media' captura la intencion de contenido (linea 1622); (2) el matcher engancha 'NOTA INFORMATIVA' por la palabra 'nota'. Distinto de P28 (que dio texto): aqui saco un recurso.</t>
         </is>
       </c>
       <c r="H56" s="21" t="inlineStr">
@@ -3411,15 +3411,15 @@
           <t>Mal</t>
         </is>
       </c>
-      <c r="E58" s="50" t="inlineStr">
-        <is>
-          <t>No aplica</t>
+      <c r="E58" s="15" t="inlineStr">
+        <is>
+          <t>Regular</t>
         </is>
       </c>
       <c r="F58" s="19" t="n"/>
       <c r="G58" s="14" t="inlineStr">
         <is>
-          <t>[SIN RE-TEST EN RONDA 3 - el veredicto de la columna Resultado es el de la evaluacion original y puede estar obsoleto] El curso no tiene actividades con nombre muy corto (&lt;=3 caracteres). No se puede probar el bug del umbral de token &gt;=4 chars. Probar en un curso con actividades tipo 'IA', 'SQL', 'T1'.</t>
+          <t>[RONDA 5 - 07/09/2026, tras v1.14.0 y v1.14.1] MEJORADO A MEDIAS. Ya NO presenta el Foro de dudas como si fuera la respuesta (antes: Mal). Ahora dice 'el documento no especifica en que consiste la actividad IA'. Pero NO dice que la actividad no existe en el curso ni ofrece las reales, que es lo que hace build_missing_activity_notice() en el caso T1.  ||  [RONDA 4 - 07/09/2026, curso SANS0001 (id 92), tras los arreglos] 'De que trata la actividad IA' (NO EXISTE en el curso) devuelve el FORO DE DUDAS. El matcher engancha un fallback arbitrario en vez de decir que no existe. Contrasta con P48, que si lo gestiona bien.  ||  El curso no tiene actividades con nombre muy corto (&lt;=3 caracteres). No se puede probar el bug del umbral de token &gt;=4 chars. Probar en un curso con actividades tipo 'IA', 'SQL', 'T1'.</t>
         </is>
       </c>
       <c r="H58" s="21" t="n"/>
@@ -3445,7 +3445,7 @@
           <t>Mal</t>
         </is>
       </c>
-      <c r="E59" s="50" t="inlineStr">
+      <c r="E59" s="49" t="inlineStr">
         <is>
           <t>No aplica</t>
         </is>
@@ -3453,7 +3453,7 @@
       <c r="F59" s="19" t="n"/>
       <c r="G59" s="14" t="inlineStr">
         <is>
-          <t>[SIN RE-TEST EN RONDA 3 - el veredicto de la columna Resultado es el de la evaluacion original y puede estar obsoleto] El curso no tiene actividades con nombre muy corto (&lt;=3 caracteres). No se puede probar el bug del umbral de token &gt;=4 chars. Probar en un curso con actividades tipo 'IA', 'SQL', 'T1'.</t>
+          <t>[RONDA 4 - 07/09/2026, curso SANS0001 (id 92), tras los arreglos] El curso no tiene ninguna seccion ni tema llamado 'SQL'. El comportamiento con nombres inexistentes queda cubierto por P46 y P48.  ||  El curso no tiene actividades con nombre muy corto (&lt;=3 caracteres). No se puede probar el bug del umbral de token &gt;=4 chars. Probar en un curso con actividades tipo 'IA', 'SQL', 'T1'.</t>
         </is>
       </c>
       <c r="H59" s="21" t="n"/>
@@ -3479,15 +3479,15 @@
           <t>Mal</t>
         </is>
       </c>
-      <c r="E60" s="50" t="inlineStr">
-        <is>
-          <t>No aplica</t>
+      <c r="E60" s="13" t="inlineStr">
+        <is>
+          <t>Bien</t>
         </is>
       </c>
       <c r="F60" s="19" t="n"/>
       <c r="G60" s="14" t="inlineStr">
         <is>
-          <t>[SIN RE-TEST EN RONDA 3 - el veredicto de la columna Resultado es el de la evaluacion original y puede estar obsoleto] El curso no tiene actividades con nombre muy corto (&lt;=3 caracteres). No se puede probar el bug del umbral de token &gt;=4 chars. Probar en un curso con actividades tipo 'IA', 'SQL', 'T1'.</t>
+          <t>[RONDA 5 - 07/09/2026, tras v1.14.0 y v1.14.1] CONFIRMADO Y MEJORADO. 'Hablame de la tarea T1': dice que no hay ninguna actividad con ese nombre y ENUMERA las actividades reales de cada seccion. Es el comportamiento que deberia tener P46.  ||  [RONDA 4 - 07/09/2026, curso SANS0001 (id 92), tras los arreglos] 'Hablame de la tarea T1' (NO EXISTE): dice que no aparece ninguna actividad con ese nombre ni ningun item de tipo assign, lista las 4 secciones reales y sugiere alternativas ('MIC Tema 1', 'MATERIAL 1'). Sin alucinar.  ||  El curso no tiene actividades con nombre muy corto (&lt;=3 caracteres). No se puede probar el bug del umbral de token &gt;=4 chars. Probar en un curso con actividades tipo 'IA', 'SQL', 'T1'.</t>
         </is>
       </c>
       <c r="H60" s="21" t="n"/>
@@ -3529,7 +3529,7 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E62" s="50" t="inlineStr">
+      <c r="E62" s="13" t="inlineStr">
         <is>
           <t>Bien</t>
         </is>
@@ -3541,7 +3541,7 @@
       </c>
       <c r="G62" s="14" t="inlineStr">
         <is>
-          <t>[SIN RE-TEST EN RONDA 3 - el veredicto de la columna Resultado es el de la evaluacion original y puede estar obsoleto] [✓ SIGUE BIEN tras fix #3: 'hazme un resumen de ese pdf' resuelve el PDF por la anafora 'ese'. (El contenido puede salir distorsionado por el bug #4 de extraccion de PDF.)]  Correcto. Valida a la vez: extraccion de texto del PDF, modo resumen (summary_mode) y history-hint ('ese pdf' resuelve el recurso mostrado antes).</t>
+          <t>[RONDA 5 - 07/09/2026, tras v1.14.0 y v1.14.1] CONFIRMADO. 'Hazme un resumen de ese pdf' tras ver MATERIAL 1 sigue resolviendo la referencia y resumiendo el contenido real.  ||  [RONDA 4 - 07/09/2026, curso SANS0001 (id 92), tras los arreglos] 'Hazme un resumen de ese pdf' tras ver MATERIAL 1: resuelve la referencia correctamente y resume el contenido real del PDF + boton de enlace. El history-hint funciona en continuaciones legitimas.  ||  [✓ SIGUE BIEN tras fix #3: 'hazme un resumen de ese pdf' resuelve el PDF por la anafora 'ese'. (El contenido puede salir distorsionado por el bug #4 de extraccion de PDF.)]  Correcto. Valida a la vez: extraccion de texto del PDF, modo resumen (summary_mode) y history-hint ('ese pdf' resuelve el recurso mostrado antes).</t>
         </is>
       </c>
       <c r="H62" s="21" t="n"/>
@@ -3567,7 +3567,7 @@
           <t>Bien</t>
         </is>
       </c>
-      <c r="E63" s="52" t="inlineStr">
+      <c r="E63" s="13" t="inlineStr">
         <is>
           <t>Bien</t>
         </is>
@@ -3579,7 +3579,7 @@
       </c>
       <c r="G63" s="14" t="inlineStr">
         <is>
-          <t>[SIN RE-TEST EN RONDA 3 - el veredicto de la columna Resultado es el de la evaluacion original y puede estar obsoleto] [✓ CONFIRMADA con fix #3 (v1.1.5): la referencia anaforica ('ese pdf'/'ese cuestionario') resuelve bien el recurso anterior; y las preguntas nuevas ya no heredan por error.]  CONFIRMADO por el usuario: el bug de contaminacion de contexto es reproducible. Ctrl+F5 (limpiar historial del cliente) lo arregla. Con contexto limpio la funcion de referencia va bien. El historial que envia el cliente contamina el matcher (history-hint). Ver P14.</t>
+          <t>[RONDA 5 - 07/09/2026, tras v1.14.0 y v1.14.1] ARREGLADO. 'Cuantas preguntas tiene ese cuestionario' tras ver el CUESTIONARIO TIPO TEST devuelve '15 preguntas' + boton de enlace. Antes repetia 'de que trata'.  ||  [RONDA 4 - 07/09/2026, curso SANS0001 (id 92), tras los arreglos] 'Cuantas preguntas tiene ese cuestionario' tras ver el CUESTIONARIO TIPO TEST devuelve DE QUE TRATA (la respuesta anterior) en vez del numero de preguntas. Contaminacion en el seguimiento; el dato si funciona en P10 (15 preguntas).  ||  [✓ CONFIRMADA con fix #3 (v1.1.5): la referencia anaforica ('ese pdf'/'ese cuestionario') resuelve bien el recurso anterior; y las preguntas nuevas ya no heredan por error.]  CONFIRMADO por el usuario: el bug de contaminacion de contexto es reproducible. Ctrl+F5 (limpiar historial del cliente) lo arregla. Con contexto limpio la funcion de referencia va bien. El historial que envia el cliente contamina el matcher (history-hint). Ver P14.</t>
         </is>
       </c>
       <c r="H63" s="21" t="n"/>
@@ -3605,7 +3605,7 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E64" s="50" t="inlineStr">
+      <c r="E64" s="16" t="inlineStr">
         <is>
           <t>Mal</t>
         </is>
@@ -3617,7 +3617,7 @@
       </c>
       <c r="G64" s="14" t="inlineStr">
         <is>
-          <t>[SIN RE-TEST EN RONDA 3 - el veredicto de la columna Resultado es el de la evaluacion original y puede estar obsoleto] Dos problemas: (1) el matcher necesita fraseo muy especifico ('el pdf X'); con fraseo suelto falla aun con contexto limpio (ver P6/P30). (2) NO soporta referencias por POSICION a documentos vistos antes ('el primero','el segundo'): las resuelve por keyword y engancha la actividad equivocada.</t>
+          <t>[RONDA 5 - 07/09/2026, tras v1.14.0 y v1.14.1] SIGUE MAL, aunque distinto. Ya no devuelve el Foro de dudas. Tras ver MATERIAL 1 y MIC Tema 2, 'dame el enunciado del primero' devuelve el enunciado de la PRIMERA PREGUNTA DEL CUESTIONARIO, ignorando los dos documentos del historial. Respuesta identica a la del mismo ordinal SIN contexto previo, lo que confirma que el ordinal no se resuelve contra el historial.  ||  [RONDA 4 - 07/09/2026, curso SANS0001 (id 92), tras los arreglos] 'Dame el enunciado del primero' tras ver MATERIAL 1 y MIC Tema 2 devuelve el FORO DE DUDAS, sin relacion con ninguno. Bug de ordinales (#5) sin resolver + fallback del matcher.  ||  Dos problemas: (1) el matcher necesita fraseo muy especifico ('el pdf X'); con fraseo suelto falla aun con contexto limpio (ver P6/P30). (2) NO soporta referencias por POSICION a documentos vistos antes ('el primero','el segundo'): las resuelve por keyword y engancha la actividad equivocada.</t>
         </is>
       </c>
       <c r="H64" s="21" t="inlineStr">
@@ -3663,9 +3663,9 @@
           <t>Mal</t>
         </is>
       </c>
-      <c r="E66" s="50" t="inlineStr">
-        <is>
-          <t>Mal</t>
+      <c r="E66" s="49" t="inlineStr">
+        <is>
+          <t>No aplica</t>
         </is>
       </c>
       <c r="F66" s="19" t="inlineStr">
@@ -3675,7 +3675,7 @@
       </c>
       <c r="G66" s="14" t="inlineStr">
         <is>
-          <t>[SIN RE-TEST EN RONDA 3 - el veredicto de la columna Resultado es el de la evaluacion original y puede estar obsoleto] El manejo de 'sin datos' es incoherente: correcto para % aprobados (P26), enganoso para nota media (por el bug de la linea 1622). Con el fix de P25 deberia dar un mensaje claro de 'sin notas'.</t>
+          <t>[RONDA 4 - 07/09/2026, curso SANS0001 (id 92), tras los arreglos] Este curso SI tiene notas (9 de 13 calificados). Haria falta un curso sin ninguna calificacion para probarlo.  ||  El manejo de 'sin datos' es incoherente: correcto para % aprobados (P26), enganoso para nota media (por el bug de la linea 1622). Con el fix de P25 deberia dar un mensaje claro de 'sin notas'.</t>
         </is>
       </c>
       <c r="H66" s="21" t="inlineStr">
@@ -3705,9 +3705,9 @@
           <t>Bien</t>
         </is>
       </c>
-      <c r="E67" s="50" t="inlineStr">
-        <is>
-          <t>Mal</t>
+      <c r="E67" s="13" t="inlineStr">
+        <is>
+          <t>Bien</t>
         </is>
       </c>
       <c r="F67" s="19" t="inlineStr">
@@ -3717,7 +3717,7 @@
       </c>
       <c r="G67" s="14" t="inlineStr">
         <is>
-          <t>[SIN RE-TEST EN RONDA 3 - el veredicto de la columna Resultado es el de la evaluacion original y puede estar obsoleto] Bloqueada por el bug del matcher (P6/P30): agarra un recurso equivocado (UF0319 vs UF0320 pedido) y no resuelve la tarea. No se puede evaluar el manejo de '0 entregas' hasta arreglar el matching. Reintentar con contexto limpio y fraseo especifico tras el fix.</t>
+          <t>[RONDA 4 - 07/09/2026, curso SANS0001 (id 92), tras los arreglos] 'Cuantas entregas hay' sin ninguna tarea en el curso: dice 0 items de tipo assign y explica que el unico calificable es un quiz. Manejo correcto del caso vacio.  ||  Bloqueada por el bug del matcher (P6/P30): agarra un recurso equivocado (UF0319 vs UF0320 pedido) y no resuelve la tarea. No se puede evaluar el manejo de '0 entregas' hasta arreglar el matching. Reintentar con contexto limpio y fraseo especifico tras el fix.</t>
         </is>
       </c>
       <c r="H67" s="21" t="inlineStr">
@@ -3805,9 +3805,9 @@
           <t>Mal</t>
         </is>
       </c>
-      <c r="E70" s="19" t="inlineStr">
-        <is>
-          <t>Mal</t>
+      <c r="E70" s="49" t="inlineStr">
+        <is>
+          <t>No aplica</t>
         </is>
       </c>
       <c r="F70" s="19" t="inlineStr">
@@ -3817,7 +3817,7 @@
       </c>
       <c r="G70" s="19" t="inlineStr">
         <is>
-          <t>[APLICADO #6.3 (v1.1.10): indexacion de contenido SCORM (lee HTML descomprimido por Moodle, orden via imsmanifest). PENDIENTE: reindexar curso y verificar 'de que trata esta unidad' sobre un SCORM HTML. Limitacion: SCORM Articulate/Storyline (JS) dara aviso claro.]  OJO: Phia y Pulso AI se probaron en CURSOS DISTINTOS (Phia en un SCORM de 'cooperativas de trabajo'; Pulso en ADGD0208 RRHH). Es una comparacion de CAPACIDAD, no de misma respuesta. Conclusion valida igualmente: Phia accede al contenido del SCORM y da objetivos de aprendizaje reales; Pulso trabaja a nivel de curso e infiere el contenido por los nombres de seccion ('probablemente/posiblemente') -&gt; riesgo de alucinacion. Para una comparacion 1:1 habria que apuntar ambos al mismo SCORM.</t>
+          <t>[RONDA 5 - 07/09/2026, tras v1.14.0 y v1.14.1] El curso SANS0001 no tiene ningun modulo SCORM (verificado: 0 enlaces a /mod/scorm/ en el curso). Segun CLAUDE.md la indexacion de SCORM sigue sin implementarse (backlog #6). Hace falta un curso con SCORM para evaluarla.  ||  [APLICADO #6.3 (v1.1.10): indexacion de contenido SCORM (lee HTML descomprimido por Moodle, orden via imsmanifest). PENDIENTE: reindexar curso y verificar 'de que trata esta unidad' sobre un SCORM HTML. Limitacion: SCORM Articulate/Storyline (JS) dara aviso claro.]  OJO: Phia y Pulso AI se probaron en CURSOS DISTINTOS (Phia en un SCORM de 'cooperativas de trabajo'; Pulso en ADGD0208 RRHH). Es una comparacion de CAPACIDAD, no de misma respuesta. Conclusion valida igualmente: Phia accede al contenido del SCORM y da objetivos de aprendizaje reales; Pulso trabaja a nivel de curso e infiere el contenido por los nombres de seccion ('probablemente/posiblemente') -&gt; riesgo de alucinacion. Para una comparacion 1:1 habria que apuntar ambos al mismo SCORM.</t>
         </is>
       </c>
       <c r="H70" s="21" t="inlineStr">
@@ -3860,9 +3860,9 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E71" s="25" t="inlineStr">
-        <is>
-          <t>Regular</t>
+      <c r="E71" s="49" t="inlineStr">
+        <is>
+          <t>No aplica</t>
         </is>
       </c>
       <c r="F71" s="19" t="inlineStr">
@@ -3872,7 +3872,7 @@
       </c>
       <c r="G71" s="19" t="inlineStr">
         <is>
-          <t>[APLICADO #6.3 (v1.1.10): mismo fix de indexacion SCORM. PENDIENTE verificar 'explicame un concepto' sobre un SCORM HTML tras reindexar.]  No falla (da explicacion valida) pero NO esta anclada en el material del curso. Para conceptos generales cuela; para conceptos con enfoque propio del curso o especificos, seria generico o podria no coincidir con lo que ensena el temario. No puede citar el material. [SEGUIMIENTO ROTO: al preguntar despues '¿cuales son los metodos mas comunes en investigacion cuantitativa?', engancho el PDF 'Principios eticos en la investigacion cientifica' por compartir 'investigacion/cientifica'. Aunque la explicacion inicial es decente, el seguimiento se rompe por el matcher (bug #2). Impide conversacion fluida sobre un tema -&gt; refuerza la prioridad del fix de P30.]</t>
+          <t>[RONDA 5 - 07/09/2026, tras v1.14.0 y v1.14.1] Igual que P55: no hay SCORM en este curso. Pendiente de un curso con SCORM.  ||  [APLICADO #6.3 (v1.1.10): mismo fix de indexacion SCORM. PENDIENTE verificar 'explicame un concepto' sobre un SCORM HTML tras reindexar.]  No falla (da explicacion valida) pero NO esta anclada en el material del curso. Para conceptos generales cuela; para conceptos con enfoque propio del curso o especificos, seria generico o podria no coincidir con lo que ensena el temario. No puede citar el material. [SEGUIMIENTO ROTO: al preguntar despues '¿cuales son los metodos mas comunes en investigacion cuantitativa?', engancho el PDF 'Principios eticos en la investigacion cientifica' por compartir 'investigacion/cientifica'. Aunque la explicacion inicial es decente, el seguimiento se rompe por el matcher (bug #2). Impide conversacion fluida sobre un tema -&gt; refuerza la prioridad del fix de P30.]</t>
         </is>
       </c>
       <c r="H71" s="21" t="inlineStr">

</xml_diff>